<commit_message>
Added columns for uniformity and glare
</commit_message>
<xml_diff>
--- a/excel/Building A B and carpark Lighting New.xlsx
+++ b/excel/Building A B and carpark Lighting New.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\310_Project1\Alpha_Design_17\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C1890B5-0704-49E0-8B49-07AA063E7017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F835CACE-7537-4F06-AA1F-FE3CCD4C11F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -26,16 +26,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="199">
   <si>
     <t>Building A — Lighting Place Schedule</t>
   </si>
@@ -626,6 +627,12 @@
   </si>
   <si>
     <t>≤ 25</t>
+  </si>
+  <si>
+    <t>Uniformity (Uo)</t>
+  </si>
+  <si>
+    <t>Glare (UGGR)</t>
   </si>
 </sst>
 </file>
@@ -1140,8 +1147,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z36"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <dimension ref="A1:AB36"/>
+  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -1154,13 +1161,13 @@
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="8.296875" customWidth="1"/>
+    <col min="17" max="17" width="8.3125" customWidth="1"/>
     <col min="18" max="20" width="12" customWidth="1"/>
     <col min="21" max="22" width="14" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21">
+    <row r="1" spans="1:28" ht="20.65">
       <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
@@ -1187,7 +1194,7 @@
       <c r="V1" s="35"/>
       <c r="W1" s="35"/>
     </row>
-    <row r="2" spans="1:26" ht="41.4">
+    <row r="2" spans="1:28" ht="41.65">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1248,26 +1255,32 @@
       <c r="T2" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="V2" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="W2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="AB2" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="27.6">
+    <row r="3" spans="1:28" ht="27">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -1324,24 +1337,26 @@
       <c r="T3" s="27" t="s">
         <v>187</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="U3" s="27"/>
+      <c r="V3" s="27"/>
+      <c r="W3" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="9"/>
-      <c r="W3" s="20"/>
-      <c r="X3" s="20" t="str">
-        <f>IF(OR(V3="",W3=""),"",V3*W3)</f>
-        <v/>
-      </c>
-      <c r="Y3" s="20" t="str">
-        <f t="shared" ref="Y3:Y36" si="1">IF(OR(S3="",X3=""),"",S3-X3)</f>
-        <v/>
-      </c>
-      <c r="Z3" s="10" t="s">
+      <c r="X3" s="9"/>
+      <c r="Y3" s="20"/>
+      <c r="Z3" s="20" t="str">
+        <f>IF(OR(X3="",Y3=""),"",X3*Y3)</f>
+        <v/>
+      </c>
+      <c r="AA3" s="20" t="str">
+        <f>IF(OR(S3="",Z3=""),"",S3-Z3)</f>
+        <v/>
+      </c>
+      <c r="AB3" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="27.6">
+    <row r="4" spans="1:28" ht="27">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -1405,24 +1420,26 @@
       <c r="T4" s="27">
         <v>503</v>
       </c>
-      <c r="U4" s="9" t="s">
+      <c r="U4" s="27"/>
+      <c r="V4" s="27"/>
+      <c r="W4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V4" s="9"/>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20" t="str">
-        <f>IF(OR(V4="",W4=""),"",V4*W4)</f>
-        <v/>
-      </c>
-      <c r="Y4" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z4" s="10" t="s">
+      <c r="X4" s="9"/>
+      <c r="Y4" s="20"/>
+      <c r="Z4" s="20" t="str">
+        <f>IF(OR(X4="",Y4=""),"",X4*Y4)</f>
+        <v/>
+      </c>
+      <c r="AA4" s="20" t="str">
+        <f>IF(OR(S4="",Z4=""),"",S4-Z4)</f>
+        <v/>
+      </c>
+      <c r="AB4" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="26.4">
+    <row r="5" spans="1:28" ht="25.5">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -1473,30 +1490,32 @@
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
       <c r="S5" s="20">
-        <f t="shared" ref="S5:S35" si="2">IF(OR(N5="",O5=""),"",N5*O5)</f>
+        <f t="shared" ref="S5:S35" si="1">IF(OR(N5="",O5=""),"",N5*O5)</f>
         <v>72</v>
       </c>
       <c r="T5" s="27">
         <v>209</v>
       </c>
-      <c r="U5" s="9" t="s">
+      <c r="U5" s="27"/>
+      <c r="V5" s="27"/>
+      <c r="W5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V5" s="9"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="20" t="str">
-        <f t="shared" ref="X5:X36" si="3">IF(OR(V5="",W5=""),"",V5*W5)</f>
-        <v/>
-      </c>
-      <c r="Y5" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z5" s="10" t="s">
+      <c r="X5" s="9"/>
+      <c r="Y5" s="20"/>
+      <c r="Z5" s="20" t="str">
+        <f t="shared" ref="Z5:Z36" si="2">IF(OR(X5="",Y5=""),"",X5*Y5)</f>
+        <v/>
+      </c>
+      <c r="AA5" s="20" t="str">
+        <f>IF(OR(S5="",Z5=""),"",S5-Z5)</f>
+        <v/>
+      </c>
+      <c r="AB5" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="26.4">
+    <row r="6" spans="1:28" ht="25.5">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -1547,30 +1566,32 @@
       <c r="Q6" s="24"/>
       <c r="R6" s="24"/>
       <c r="S6" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="T6" s="27">
         <v>209</v>
       </c>
-      <c r="U6" s="9" t="s">
+      <c r="U6" s="27"/>
+      <c r="V6" s="27"/>
+      <c r="W6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V6" s="9"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y6" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z6" s="10" t="s">
+      <c r="X6" s="9"/>
+      <c r="Y6" s="20"/>
+      <c r="Z6" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA6" s="20" t="str">
+        <f>IF(OR(S6="",Z6=""),"",S6-Z6)</f>
+        <v/>
+      </c>
+      <c r="AB6" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="26.4">
+    <row r="7" spans="1:28" ht="25.5">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -1621,30 +1642,32 @@
       <c r="Q7" s="24"/>
       <c r="R7" s="24"/>
       <c r="S7" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="T7" s="27">
         <v>183</v>
       </c>
-      <c r="U7" s="9" t="s">
+      <c r="U7" s="27"/>
+      <c r="V7" s="27"/>
+      <c r="W7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V7" s="9"/>
-      <c r="W7" s="20"/>
-      <c r="X7" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y7" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z7" s="10" t="s">
+      <c r="X7" s="9"/>
+      <c r="Y7" s="20"/>
+      <c r="Z7" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA7" s="20" t="str">
+        <f>IF(OR(S7="",Z7=""),"",S7-Z7)</f>
+        <v/>
+      </c>
+      <c r="AB7" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="26.4">
+    <row r="8" spans="1:28" ht="25.5">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -1695,30 +1718,32 @@
       <c r="Q8" s="24"/>
       <c r="R8" s="24"/>
       <c r="S8" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>288</v>
       </c>
       <c r="T8" s="27">
         <v>625</v>
       </c>
-      <c r="U8" s="9" t="s">
+      <c r="U8" s="27"/>
+      <c r="V8" s="27"/>
+      <c r="W8" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V8" s="9"/>
-      <c r="W8" s="20"/>
-      <c r="X8" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y8" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z8" s="10" t="s">
+      <c r="X8" s="9"/>
+      <c r="Y8" s="20"/>
+      <c r="Z8" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA8" s="20" t="str">
+        <f>IF(OR(S8="",Z8=""),"",S8-Z8)</f>
+        <v/>
+      </c>
+      <c r="AB8" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="26.4">
+    <row r="9" spans="1:28" ht="25.5">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -1769,30 +1794,32 @@
       <c r="Q9" s="24"/>
       <c r="R9" s="24"/>
       <c r="S9" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>288</v>
       </c>
       <c r="T9" s="27">
         <v>644</v>
       </c>
-      <c r="U9" s="9" t="s">
+      <c r="U9" s="27"/>
+      <c r="V9" s="27"/>
+      <c r="W9" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V9" s="9"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y9" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z9" s="10" t="s">
+      <c r="X9" s="9"/>
+      <c r="Y9" s="20"/>
+      <c r="Z9" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA9" s="20" t="str">
+        <f>IF(OR(S9="",Z9=""),"",S9-Z9)</f>
+        <v/>
+      </c>
+      <c r="AB9" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="27.6">
+    <row r="10" spans="1:28" ht="27">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1856,24 +1883,26 @@
       <c r="T10" s="27">
         <v>373</v>
       </c>
-      <c r="U10" s="9" t="s">
+      <c r="U10" s="27"/>
+      <c r="V10" s="27"/>
+      <c r="W10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V10" s="9"/>
-      <c r="W10" s="20"/>
-      <c r="X10" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y10" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z10" s="10" t="s">
+      <c r="X10" s="9"/>
+      <c r="Y10" s="20"/>
+      <c r="Z10" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA10" s="20" t="str">
+        <f>IF(OR(S10="",Z10=""),"",S10-Z10)</f>
+        <v/>
+      </c>
+      <c r="AB10" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="26.4">
+    <row r="11" spans="1:28" ht="25.5">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -1924,29 +1953,31 @@
       <c r="Q11" s="24"/>
       <c r="R11" s="24"/>
       <c r="S11" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>288</v>
       </c>
       <c r="T11" s="27">
         <v>615</v>
       </c>
-      <c r="U11" s="9" t="s">
+      <c r="U11" s="27"/>
+      <c r="V11" s="27"/>
+      <c r="W11" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="W11" s="20"/>
-      <c r="X11" s="20" t="str">
-        <f>IF(OR(V12="",W11=""),"",V12*W11)</f>
-        <v/>
-      </c>
-      <c r="Y11" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z11" s="10" t="s">
+      <c r="Y11" s="20"/>
+      <c r="Z11" s="20" t="str">
+        <f>IF(OR(X12="",Y11=""),"",X12*Y11)</f>
+        <v/>
+      </c>
+      <c r="AA11" s="20" t="str">
+        <f>IF(OR(S11="",Z11=""),"",S11-Z11)</f>
+        <v/>
+      </c>
+      <c r="AB11" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="26.4">
+    <row r="12" spans="1:28" ht="25.5">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -1997,30 +2028,32 @@
       <c r="Q12" s="24"/>
       <c r="R12" s="24"/>
       <c r="S12" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T12" s="27">
         <v>836</v>
       </c>
-      <c r="U12" s="9" t="s">
+      <c r="U12" s="27"/>
+      <c r="V12" s="27"/>
+      <c r="W12" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V12" s="9"/>
-      <c r="W12" s="20"/>
-      <c r="X12" s="20" t="e">
-        <f>IF(OR(#REF!="",W12=""),"",#REF!*W12)</f>
+      <c r="X12" s="9"/>
+      <c r="Y12" s="20"/>
+      <c r="Z12" s="20" t="e">
+        <f>IF(OR(#REF!="",Y12=""),"",#REF!*Y12)</f>
         <v>#REF!</v>
       </c>
-      <c r="Y12" s="20" t="e">
-        <f t="shared" si="1"/>
+      <c r="AA12" s="20" t="e">
+        <f>IF(OR(S12="",Z12=""),"",S12-Z12)</f>
         <v>#REF!</v>
       </c>
-      <c r="Z12" s="10" t="s">
+      <c r="AB12" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="26.4">
+    <row r="13" spans="1:28" ht="25.5">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -2071,30 +2104,32 @@
       <c r="Q13" s="24"/>
       <c r="R13" s="24"/>
       <c r="S13" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T13" s="27">
         <v>743</v>
       </c>
-      <c r="U13" s="9" t="s">
+      <c r="U13" s="27"/>
+      <c r="V13" s="27"/>
+      <c r="W13" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V13" s="9"/>
-      <c r="W13" s="20"/>
-      <c r="X13" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y13" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z13" s="10" t="s">
+      <c r="X13" s="9"/>
+      <c r="Y13" s="20"/>
+      <c r="Z13" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA13" s="20" t="str">
+        <f>IF(OR(S13="",Z13=""),"",S13-Z13)</f>
+        <v/>
+      </c>
+      <c r="AB13" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="26.4">
+    <row r="14" spans="1:28" ht="25.5">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -2145,30 +2180,32 @@
       <c r="Q14" s="24"/>
       <c r="R14" s="24"/>
       <c r="S14" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>864</v>
       </c>
       <c r="T14" s="27">
         <v>1088</v>
       </c>
-      <c r="U14" s="9" t="s">
+      <c r="U14" s="27"/>
+      <c r="V14" s="27"/>
+      <c r="W14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V14" s="9"/>
-      <c r="W14" s="20"/>
-      <c r="X14" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y14" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z14" s="10" t="s">
+      <c r="X14" s="9"/>
+      <c r="Y14" s="20"/>
+      <c r="Z14" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA14" s="20" t="str">
+        <f>IF(OR(S14="",Z14=""),"",S14-Z14)</f>
+        <v/>
+      </c>
+      <c r="AB14" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="26.4">
+    <row r="15" spans="1:28" ht="25.5">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -2219,30 +2256,32 @@
       <c r="Q15" s="24"/>
       <c r="R15" s="24"/>
       <c r="S15" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>432</v>
       </c>
       <c r="T15" s="27">
         <v>743</v>
       </c>
-      <c r="U15" s="9" t="s">
+      <c r="U15" s="27"/>
+      <c r="V15" s="27"/>
+      <c r="W15" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V15" s="9"/>
-      <c r="W15" s="20"/>
-      <c r="X15" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y15" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z15" s="10" t="s">
+      <c r="X15" s="9"/>
+      <c r="Y15" s="20"/>
+      <c r="Z15" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA15" s="20" t="str">
+        <f>IF(OR(S15="",Z15=""),"",S15-Z15)</f>
+        <v/>
+      </c>
+      <c r="AB15" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="26.4">
+    <row r="16" spans="1:28" ht="25.5">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2293,30 +2332,32 @@
       <c r="Q16" s="24"/>
       <c r="R16" s="24"/>
       <c r="S16" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>432</v>
       </c>
       <c r="T16" s="27">
         <v>954</v>
       </c>
-      <c r="U16" s="9" t="s">
+      <c r="U16" s="27"/>
+      <c r="V16" s="27"/>
+      <c r="W16" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V16" s="9"/>
-      <c r="W16" s="20"/>
-      <c r="X16" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y16" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z16" s="10" t="s">
+      <c r="X16" s="9"/>
+      <c r="Y16" s="20"/>
+      <c r="Z16" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA16" s="20" t="str">
+        <f>IF(OR(S16="",Z16=""),"",S16-Z16)</f>
+        <v/>
+      </c>
+      <c r="AB16" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:26" ht="27.6">
+    <row r="17" spans="1:28" ht="27">
       <c r="A17" s="6" t="s">
         <v>78</v>
       </c>
@@ -2367,30 +2408,32 @@
       <c r="Q17" s="24"/>
       <c r="R17" s="24"/>
       <c r="S17" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="T17" s="27">
         <v>150</v>
       </c>
-      <c r="U17" s="9" t="s">
+      <c r="U17" s="27"/>
+      <c r="V17" s="27"/>
+      <c r="W17" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V17" s="9"/>
-      <c r="W17" s="20"/>
-      <c r="X17" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y17" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z17" s="10" t="s">
+      <c r="X17" s="9"/>
+      <c r="Y17" s="20"/>
+      <c r="Z17" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA17" s="20" t="str">
+        <f>IF(OR(S17="",Z17=""),"",S17-Z17)</f>
+        <v/>
+      </c>
+      <c r="AB17" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:26" ht="27.6">
+    <row r="18" spans="1:28" ht="27">
       <c r="A18" s="6" t="s">
         <v>78</v>
       </c>
@@ -2441,30 +2484,32 @@
       <c r="Q18" s="24"/>
       <c r="R18" s="24"/>
       <c r="S18" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>288</v>
       </c>
       <c r="T18" s="27">
         <v>140</v>
       </c>
-      <c r="U18" s="9" t="s">
+      <c r="U18" s="27"/>
+      <c r="V18" s="27"/>
+      <c r="W18" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V18" s="9"/>
-      <c r="W18" s="20"/>
-      <c r="X18" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y18" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z18" s="10" t="s">
+      <c r="X18" s="9"/>
+      <c r="Y18" s="20"/>
+      <c r="Z18" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA18" s="20" t="str">
+        <f>IF(OR(S18="",Z18=""),"",S18-Z18)</f>
+        <v/>
+      </c>
+      <c r="AB18" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:26" ht="26.4">
+    <row r="19" spans="1:28" ht="25.5">
       <c r="A19" s="6" t="s">
         <v>78</v>
       </c>
@@ -2515,30 +2560,32 @@
       <c r="Q19" s="24"/>
       <c r="R19" s="24"/>
       <c r="S19" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>288</v>
       </c>
       <c r="T19" s="27">
         <v>331</v>
       </c>
-      <c r="U19" s="9" t="s">
+      <c r="U19" s="27"/>
+      <c r="V19" s="27"/>
+      <c r="W19" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V19" s="9"/>
-      <c r="W19" s="20"/>
-      <c r="X19" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y19" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z19" s="10" t="s">
+      <c r="X19" s="9"/>
+      <c r="Y19" s="20"/>
+      <c r="Z19" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA19" s="20" t="str">
+        <f>IF(OR(S19="",Z19=""),"",S19-Z19)</f>
+        <v/>
+      </c>
+      <c r="AB19" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:26" ht="26.4">
+    <row r="20" spans="1:28" ht="25.5">
       <c r="A20" s="6" t="s">
         <v>78</v>
       </c>
@@ -2589,30 +2636,32 @@
       <c r="Q20" s="24"/>
       <c r="R20" s="24"/>
       <c r="S20" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1008</v>
       </c>
       <c r="T20" s="27">
         <v>470</v>
       </c>
-      <c r="U20" s="9" t="s">
+      <c r="U20" s="27"/>
+      <c r="V20" s="27"/>
+      <c r="W20" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V20" s="9"/>
-      <c r="W20" s="20"/>
-      <c r="X20" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y20" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z20" s="10" t="s">
+      <c r="X20" s="9"/>
+      <c r="Y20" s="20"/>
+      <c r="Z20" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA20" s="20" t="str">
+        <f>IF(OR(S20="",Z20=""),"",S20-Z20)</f>
+        <v/>
+      </c>
+      <c r="AB20" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:26" ht="27.6">
+    <row r="21" spans="1:28" ht="27">
       <c r="A21" s="6" t="s">
         <v>78</v>
       </c>
@@ -2663,30 +2712,32 @@
       <c r="Q21" s="24"/>
       <c r="R21" s="24"/>
       <c r="S21" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="T21" s="27">
         <v>181</v>
       </c>
-      <c r="U21" s="9" t="s">
+      <c r="U21" s="27"/>
+      <c r="V21" s="27"/>
+      <c r="W21" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V21" s="9"/>
-      <c r="W21" s="20"/>
-      <c r="X21" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y21" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z21" s="10" t="s">
+      <c r="X21" s="9"/>
+      <c r="Y21" s="20"/>
+      <c r="Z21" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA21" s="20" t="str">
+        <f>IF(OR(S21="",Z21=""),"",S21-Z21)</f>
+        <v/>
+      </c>
+      <c r="AB21" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:26" ht="26.4">
+    <row r="22" spans="1:28" ht="25.5">
       <c r="A22" s="6" t="s">
         <v>78</v>
       </c>
@@ -2737,30 +2788,32 @@
       <c r="Q22" s="24"/>
       <c r="R22" s="24"/>
       <c r="S22" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>144</v>
       </c>
       <c r="T22" s="27">
         <v>269</v>
       </c>
-      <c r="U22" s="9" t="s">
+      <c r="U22" s="27"/>
+      <c r="V22" s="27"/>
+      <c r="W22" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V22" s="9"/>
-      <c r="W22" s="20"/>
-      <c r="X22" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y22" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z22" s="10" t="s">
+      <c r="X22" s="9"/>
+      <c r="Y22" s="20"/>
+      <c r="Z22" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA22" s="20" t="str">
+        <f>IF(OR(S22="",Z22=""),"",S22-Z22)</f>
+        <v/>
+      </c>
+      <c r="AB22" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:26" ht="26.4">
+    <row r="23" spans="1:28" ht="25.5">
       <c r="A23" s="6" t="s">
         <v>78</v>
       </c>
@@ -2811,30 +2864,32 @@
       <c r="Q23" s="24"/>
       <c r="R23" s="24"/>
       <c r="S23" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>864</v>
       </c>
       <c r="T23" s="27">
         <v>516</v>
       </c>
-      <c r="U23" s="9" t="s">
+      <c r="U23" s="27"/>
+      <c r="V23" s="27"/>
+      <c r="W23" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V23" s="9"/>
-      <c r="W23" s="20"/>
-      <c r="X23" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y23" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z23" s="10" t="s">
+      <c r="X23" s="9"/>
+      <c r="Y23" s="20"/>
+      <c r="Z23" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA23" s="20" t="str">
+        <f>IF(OR(S23="",Z23=""),"",S23-Z23)</f>
+        <v/>
+      </c>
+      <c r="AB23" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:26" ht="26.4">
+    <row r="24" spans="1:28" ht="25.5">
       <c r="A24" s="6" t="s">
         <v>78</v>
       </c>
@@ -2885,30 +2940,32 @@
       <c r="Q24" s="24"/>
       <c r="R24" s="24"/>
       <c r="S24" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T24" s="27">
         <v>458</v>
       </c>
-      <c r="U24" s="9" t="s">
+      <c r="U24" s="27"/>
+      <c r="V24" s="27"/>
+      <c r="W24" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V24" s="9"/>
-      <c r="W24" s="20"/>
-      <c r="X24" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y24" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z24" s="10" t="s">
+      <c r="X24" s="9"/>
+      <c r="Y24" s="20"/>
+      <c r="Z24" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA24" s="20" t="str">
+        <f>IF(OR(S24="",Z24=""),"",S24-Z24)</f>
+        <v/>
+      </c>
+      <c r="AB24" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="26.4">
+    <row r="25" spans="1:28" ht="25.5">
       <c r="A25" s="6" t="s">
         <v>78</v>
       </c>
@@ -2959,30 +3016,32 @@
       <c r="Q25" s="24"/>
       <c r="R25" s="24"/>
       <c r="S25" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T25" s="27">
         <v>422</v>
       </c>
-      <c r="U25" s="9" t="s">
+      <c r="U25" s="27"/>
+      <c r="V25" s="27"/>
+      <c r="W25" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V25" s="9"/>
-      <c r="W25" s="20"/>
-      <c r="X25" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y25" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z25" s="10" t="s">
+      <c r="X25" s="9"/>
+      <c r="Y25" s="20"/>
+      <c r="Z25" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA25" s="20" t="str">
+        <f>IF(OR(S25="",Z25=""),"",S25-Z25)</f>
+        <v/>
+      </c>
+      <c r="AB25" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:26" ht="26.4">
+    <row r="26" spans="1:28" ht="25.5">
       <c r="A26" s="6" t="s">
         <v>78</v>
       </c>
@@ -3033,30 +3092,32 @@
       <c r="Q26" s="24"/>
       <c r="R26" s="24"/>
       <c r="S26" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1152</v>
       </c>
       <c r="T26" s="27">
         <v>455</v>
       </c>
-      <c r="U26" s="9" t="s">
+      <c r="U26" s="27"/>
+      <c r="V26" s="27"/>
+      <c r="W26" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V26" s="9"/>
-      <c r="W26" s="20"/>
-      <c r="X26" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y26" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z26" s="10" t="s">
+      <c r="X26" s="9"/>
+      <c r="Y26" s="20"/>
+      <c r="Z26" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA26" s="20" t="str">
+        <f>IF(OR(S26="",Z26=""),"",S26-Z26)</f>
+        <v/>
+      </c>
+      <c r="AB26" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:26" ht="27.6">
+    <row r="27" spans="1:28" ht="27">
       <c r="A27" s="6" t="s">
         <v>78</v>
       </c>
@@ -3107,30 +3168,32 @@
       <c r="Q27" s="24"/>
       <c r="R27" s="24"/>
       <c r="S27" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T27" s="27">
         <v>133</v>
       </c>
-      <c r="U27" s="9" t="s">
+      <c r="U27" s="27"/>
+      <c r="V27" s="27"/>
+      <c r="W27" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V27" s="9"/>
-      <c r="W27" s="20"/>
-      <c r="X27" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y27" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z27" s="10" t="s">
+      <c r="X27" s="9"/>
+      <c r="Y27" s="20"/>
+      <c r="Z27" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA27" s="20" t="str">
+        <f>IF(OR(S27="",Z27=""),"",S27-Z27)</f>
+        <v/>
+      </c>
+      <c r="AB27" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:26" ht="26.4">
+    <row r="28" spans="1:28" ht="25.5">
       <c r="A28" s="6" t="s">
         <v>78</v>
       </c>
@@ -3181,30 +3244,32 @@
       <c r="Q28" s="24"/>
       <c r="R28" s="24"/>
       <c r="S28" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1152</v>
       </c>
       <c r="T28" s="27">
         <v>435</v>
       </c>
-      <c r="U28" s="9" t="s">
+      <c r="U28" s="27"/>
+      <c r="V28" s="27"/>
+      <c r="W28" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V28" s="9"/>
-      <c r="W28" s="20"/>
-      <c r="X28" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y28" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z28" s="10" t="s">
+      <c r="X28" s="9"/>
+      <c r="Y28" s="20"/>
+      <c r="Z28" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA28" s="20" t="str">
+        <f>IF(OR(S28="",Z28=""),"",S28-Z28)</f>
+        <v/>
+      </c>
+      <c r="AB28" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:26" ht="27.6">
+    <row r="29" spans="1:28" ht="27">
       <c r="A29" s="6" t="s">
         <v>78</v>
       </c>
@@ -3255,30 +3320,32 @@
       <c r="Q29" s="24"/>
       <c r="R29" s="24"/>
       <c r="S29" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="T29" s="27">
         <v>118</v>
       </c>
-      <c r="U29" s="9" t="s">
+      <c r="U29" s="27"/>
+      <c r="V29" s="27"/>
+      <c r="W29" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V29" s="9"/>
-      <c r="W29" s="20"/>
-      <c r="X29" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y29" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z29" s="10" t="s">
+      <c r="X29" s="9"/>
+      <c r="Y29" s="20"/>
+      <c r="Z29" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA29" s="20" t="str">
+        <f>IF(OR(S29="",Z29=""),"",S29-Z29)</f>
+        <v/>
+      </c>
+      <c r="AB29" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:26" ht="26.4">
+    <row r="30" spans="1:28" ht="25.5">
       <c r="A30" s="6" t="s">
         <v>78</v>
       </c>
@@ -3329,30 +3396,32 @@
       <c r="Q30" s="24"/>
       <c r="R30" s="24"/>
       <c r="S30" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T30" s="27">
         <v>416</v>
       </c>
-      <c r="U30" s="9" t="s">
+      <c r="U30" s="27"/>
+      <c r="V30" s="27"/>
+      <c r="W30" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V30" s="9"/>
-      <c r="W30" s="20"/>
-      <c r="X30" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y30" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z30" s="10" t="s">
+      <c r="X30" s="9"/>
+      <c r="Y30" s="20"/>
+      <c r="Z30" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA30" s="20" t="str">
+        <f>IF(OR(S30="",Z30=""),"",S30-Z30)</f>
+        <v/>
+      </c>
+      <c r="AB30" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:26" ht="26.4">
+    <row r="31" spans="1:28" ht="25.5">
       <c r="A31" s="6" t="s">
         <v>78</v>
       </c>
@@ -3403,30 +3472,32 @@
       <c r="Q31" s="24"/>
       <c r="R31" s="24"/>
       <c r="S31" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T31" s="27">
         <v>419</v>
       </c>
-      <c r="U31" s="9" t="s">
+      <c r="U31" s="27"/>
+      <c r="V31" s="27"/>
+      <c r="W31" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V31" s="9"/>
-      <c r="W31" s="20"/>
-      <c r="X31" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y31" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z31" s="10" t="s">
+      <c r="X31" s="9"/>
+      <c r="Y31" s="20"/>
+      <c r="Z31" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA31" s="20" t="str">
+        <f>IF(OR(S31="",Z31=""),"",S31-Z31)</f>
+        <v/>
+      </c>
+      <c r="AB31" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:26" ht="26.4">
+    <row r="32" spans="1:28" ht="25.5">
       <c r="A32" s="6" t="s">
         <v>78</v>
       </c>
@@ -3477,30 +3548,32 @@
       <c r="Q32" s="24"/>
       <c r="R32" s="24"/>
       <c r="S32" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>576</v>
       </c>
       <c r="T32" s="27">
         <v>400</v>
       </c>
-      <c r="U32" s="9" t="s">
+      <c r="U32" s="27"/>
+      <c r="V32" s="27"/>
+      <c r="W32" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V32" s="9"/>
-      <c r="W32" s="20"/>
-      <c r="X32" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y32" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z32" s="10" t="s">
+      <c r="X32" s="9"/>
+      <c r="Y32" s="20"/>
+      <c r="Z32" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA32" s="20" t="str">
+        <f>IF(OR(S32="",Z32=""),"",S32-Z32)</f>
+        <v/>
+      </c>
+      <c r="AB32" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:26" ht="26.4">
+    <row r="33" spans="1:28" ht="25.5">
       <c r="A33" s="6" t="s">
         <v>78</v>
       </c>
@@ -3551,30 +3624,32 @@
       <c r="Q33" s="24"/>
       <c r="R33" s="24"/>
       <c r="S33" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="T33" s="27">
         <v>140</v>
       </c>
-      <c r="U33" s="9" t="s">
+      <c r="U33" s="27"/>
+      <c r="V33" s="27"/>
+      <c r="W33" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V33" s="9"/>
-      <c r="W33" s="20"/>
-      <c r="X33" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y33" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z33" s="10" t="s">
+      <c r="X33" s="9"/>
+      <c r="Y33" s="20"/>
+      <c r="Z33" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA33" s="20" t="str">
+        <f>IF(OR(S33="",Z33=""),"",S33-Z33)</f>
+        <v/>
+      </c>
+      <c r="AB33" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:26" ht="26.4">
+    <row r="34" spans="1:28" ht="25.5">
       <c r="A34" s="6" t="s">
         <v>78</v>
       </c>
@@ -3625,30 +3700,32 @@
       <c r="Q34" s="24"/>
       <c r="R34" s="24"/>
       <c r="S34" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="T34" s="27">
         <v>140</v>
       </c>
-      <c r="U34" s="9" t="s">
+      <c r="U34" s="27"/>
+      <c r="V34" s="27"/>
+      <c r="W34" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V34" s="9"/>
-      <c r="W34" s="20"/>
-      <c r="X34" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y34" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z34" s="10" t="s">
+      <c r="X34" s="9"/>
+      <c r="Y34" s="20"/>
+      <c r="Z34" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA34" s="20" t="str">
+        <f>IF(OR(S34="",Z34=""),"",S34-Z34)</f>
+        <v/>
+      </c>
+      <c r="AB34" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:26" ht="26.4">
+    <row r="35" spans="1:28" ht="25.5">
       <c r="A35" s="6" t="s">
         <v>78</v>
       </c>
@@ -3699,30 +3776,32 @@
       <c r="Q35" s="24"/>
       <c r="R35" s="24"/>
       <c r="S35" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>432</v>
       </c>
       <c r="T35" s="27">
         <v>405</v>
       </c>
-      <c r="U35" s="9" t="s">
+      <c r="U35" s="27"/>
+      <c r="V35" s="27"/>
+      <c r="W35" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V35" s="9"/>
-      <c r="W35" s="20"/>
-      <c r="X35" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y35" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z35" s="10" t="s">
+      <c r="X35" s="9"/>
+      <c r="Y35" s="20"/>
+      <c r="Z35" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA35" s="20" t="str">
+        <f>IF(OR(S35="",Z35=""),"",S35-Z35)</f>
+        <v/>
+      </c>
+      <c r="AB35" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="26.4">
+    <row r="36" spans="1:28" ht="25.5">
       <c r="A36" s="11" t="s">
         <v>78</v>
       </c>
@@ -3779,20 +3858,22 @@
       <c r="T36" s="27">
         <v>392</v>
       </c>
-      <c r="U36" s="14" t="s">
+      <c r="U36" s="27"/>
+      <c r="V36" s="27"/>
+      <c r="W36" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="V36" s="14"/>
-      <c r="W36" s="21"/>
-      <c r="X36" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="Y36" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="Z36" s="15" t="s">
+      <c r="X36" s="14"/>
+      <c r="Y36" s="21"/>
+      <c r="Z36" s="21" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="AA36" s="21" t="str">
+        <f>IF(OR(S36="",Z36=""),"",S36-Z36)</f>
+        <v/>
+      </c>
+      <c r="AB36" s="15" t="s">
         <v>31</v>
       </c>
     </row>
@@ -3800,7 +3881,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:W1"/>
   </mergeCells>
-  <conditionalFormatting sqref="T4:T36">
+  <conditionalFormatting sqref="T4:V36">
     <cfRule type="expression" dxfId="5" priority="1">
       <formula>$T4&lt;$F4</formula>
     </cfRule>
@@ -3815,8 +3896,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z41"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <dimension ref="A1:AB41"/>
+  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -3829,7 +3910,7 @@
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="15.69921875" customWidth="1"/>
+    <col min="17" max="17" width="15.6875" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="20" width="14" customWidth="1"/>
     <col min="21" max="21" width="24" customWidth="1"/>
@@ -3838,7 +3919,7 @@
     <col min="26" max="26" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21">
+    <row r="1" spans="1:28" ht="20.65">
       <c r="A1" s="35" t="s">
         <v>105</v>
       </c>
@@ -3868,7 +3949,7 @@
       <c r="Y1" s="35"/>
       <c r="Z1" s="35"/>
     </row>
-    <row r="2" spans="1:26" ht="41.4">
+    <row r="2" spans="1:28" ht="41.65">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -3929,26 +4010,32 @@
       <c r="T2" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="V2" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="W2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="AB2" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="26.4">
+    <row r="3" spans="1:28" ht="25.5">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -4013,24 +4100,26 @@
       <c r="T3" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="U3" s="27"/>
+      <c r="V3" s="27"/>
+      <c r="W3" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="9"/>
-      <c r="W3" s="20"/>
-      <c r="X3" s="20" t="str">
-        <f t="shared" ref="X3:X24" si="1">IF(OR(V3="",W3=""),"",V3*W3)</f>
-        <v/>
-      </c>
-      <c r="Y3" s="20" t="str">
-        <f t="shared" ref="Y3:Y24" si="2">IF(OR(S3="",X3=""),"",S3-X3)</f>
-        <v/>
-      </c>
-      <c r="Z3" s="10" t="s">
+      <c r="X3" s="9"/>
+      <c r="Y3" s="20"/>
+      <c r="Z3" s="20" t="str">
+        <f t="shared" ref="Z3:Z24" si="1">IF(OR(X3="",Y3=""),"",X3*Y3)</f>
+        <v/>
+      </c>
+      <c r="AA3" s="20" t="str">
+        <f>IF(OR(S3="",Z3=""),"",S3-Z3)</f>
+        <v/>
+      </c>
+      <c r="AB3" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="26.4">
+    <row r="4" spans="1:28" ht="25.5">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -4075,7 +4164,7 @@
         <v>2</v>
       </c>
       <c r="O4" s="20">
-        <f t="shared" ref="O4:O23" si="3">2*36*N4</f>
+        <f t="shared" ref="O4:O23" si="2">2*36*N4</f>
         <v>144</v>
       </c>
       <c r="P4" s="25" t="s">
@@ -4085,34 +4174,36 @@
         <v>5</v>
       </c>
       <c r="R4" s="24">
-        <f t="shared" ref="R4:R24" si="4">4*36*Q4</f>
+        <f t="shared" ref="R4:R24" si="3">4*36*Q4</f>
         <v>720</v>
       </c>
       <c r="S4" s="20">
-        <f t="shared" ref="S4:S23" si="5">O4+R4</f>
+        <f t="shared" ref="S4:S23" si="4">O4+R4</f>
         <v>864</v>
       </c>
       <c r="T4" s="27">
         <v>380</v>
       </c>
-      <c r="U4" s="9" t="s">
+      <c r="U4" s="27"/>
+      <c r="V4" s="27"/>
+      <c r="W4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V4" s="9"/>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20" t="str">
+      <c r="X4" s="9"/>
+      <c r="Y4" s="20"/>
+      <c r="Z4" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y4" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z4" s="10" t="s">
+      <c r="AA4" s="20" t="str">
+        <f>IF(OR(S4="",Z4=""),"",S4-Z4)</f>
+        <v/>
+      </c>
+      <c r="AB4" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="26.4">
+    <row r="5" spans="1:28" ht="25.5">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -4157,7 +4248,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P5" s="25" t="s">
@@ -4167,34 +4258,36 @@
         <v>1</v>
       </c>
       <c r="R5" s="24">
+        <f t="shared" si="3"/>
+        <v>144</v>
+      </c>
+      <c r="S5" s="20">
         <f t="shared" si="4"/>
         <v>144</v>
       </c>
-      <c r="S5" s="20">
-        <f t="shared" si="5"/>
-        <v>144</v>
-      </c>
       <c r="T5" s="27">
         <v>325</v>
       </c>
-      <c r="U5" s="9" t="s">
+      <c r="U5" s="27"/>
+      <c r="V5" s="27"/>
+      <c r="W5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V5" s="9"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="20" t="str">
+      <c r="X5" s="9"/>
+      <c r="Y5" s="20"/>
+      <c r="Z5" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y5" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z5" s="10" t="s">
+      <c r="AA5" s="20" t="str">
+        <f>IF(OR(S5="",Z5=""),"",S5-Z5)</f>
+        <v/>
+      </c>
+      <c r="AB5" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="26.4">
+    <row r="6" spans="1:28" ht="25.5">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -4239,7 +4332,7 @@
         <v>1</v>
       </c>
       <c r="O6" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="P6" s="25" t="s">
@@ -4249,34 +4342,36 @@
         <v>0</v>
       </c>
       <c r="R6" s="24">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S6" s="20">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S6" s="20">
-        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T6" s="27">
         <v>205</v>
       </c>
-      <c r="U6" s="9" t="s">
+      <c r="U6" s="27"/>
+      <c r="V6" s="27"/>
+      <c r="W6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V6" s="9"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20" t="str">
+      <c r="X6" s="9"/>
+      <c r="Y6" s="20"/>
+      <c r="Z6" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y6" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z6" s="10" t="s">
+      <c r="AA6" s="20" t="str">
+        <f>IF(OR(S6="",Z6=""),"",S6-Z6)</f>
+        <v/>
+      </c>
+      <c r="AB6" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="26.4">
+    <row r="7" spans="1:28" ht="25.5">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -4321,7 +4416,7 @@
         <v>1</v>
       </c>
       <c r="O7" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="P7" s="25" t="s">
@@ -4331,34 +4426,36 @@
         <v>0</v>
       </c>
       <c r="R7" s="24">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S7" s="20">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S7" s="20">
-        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T7" s="27">
         <v>201</v>
       </c>
-      <c r="U7" s="9" t="s">
+      <c r="U7" s="27"/>
+      <c r="V7" s="27"/>
+      <c r="W7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V7" s="9"/>
-      <c r="W7" s="20"/>
-      <c r="X7" s="20" t="str">
+      <c r="X7" s="9"/>
+      <c r="Y7" s="20"/>
+      <c r="Z7" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y7" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z7" s="10" t="s">
+      <c r="AA7" s="20" t="str">
+        <f>IF(OR(S7="",Z7=""),"",S7-Z7)</f>
+        <v/>
+      </c>
+      <c r="AB7" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="26.4">
+    <row r="8" spans="1:28" ht="25.5">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -4403,7 +4500,7 @@
         <v>1</v>
       </c>
       <c r="O8" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="P8" s="25" t="s">
@@ -4413,34 +4510,36 @@
         <v>0</v>
       </c>
       <c r="R8" s="24">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S8" s="20">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S8" s="20">
-        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T8" s="27">
         <v>186</v>
       </c>
-      <c r="U8" s="9" t="s">
+      <c r="U8" s="27"/>
+      <c r="V8" s="27"/>
+      <c r="W8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V8" s="9"/>
-      <c r="W8" s="20"/>
-      <c r="X8" s="20" t="str">
+      <c r="X8" s="9"/>
+      <c r="Y8" s="20"/>
+      <c r="Z8" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y8" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z8" s="10" t="s">
+      <c r="AA8" s="20" t="str">
+        <f>IF(OR(S8="",Z8=""),"",S8-Z8)</f>
+        <v/>
+      </c>
+      <c r="AB8" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="26.4">
+    <row r="9" spans="1:28" ht="25.5">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -4485,7 +4584,7 @@
         <v>1</v>
       </c>
       <c r="O9" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="P9" s="25" t="s">
@@ -4495,34 +4594,36 @@
         <v>0</v>
       </c>
       <c r="R9" s="24">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S9" s="20">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S9" s="20">
-        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T9" s="27">
         <v>187</v>
       </c>
-      <c r="U9" s="9" t="s">
+      <c r="U9" s="27"/>
+      <c r="V9" s="27"/>
+      <c r="W9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V9" s="9"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="20" t="str">
+      <c r="X9" s="9"/>
+      <c r="Y9" s="20"/>
+      <c r="Z9" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y9" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z9" s="10" t="s">
+      <c r="AA9" s="20" t="str">
+        <f>IF(OR(S9="",Z9=""),"",S9-Z9)</f>
+        <v/>
+      </c>
+      <c r="AB9" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="26.4">
+    <row r="10" spans="1:28" ht="25.5">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -4567,7 +4668,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P10" s="25" t="s">
@@ -4577,34 +4678,36 @@
         <v>4</v>
       </c>
       <c r="R10" s="24">
+        <f t="shared" si="3"/>
+        <v>576</v>
+      </c>
+      <c r="S10" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
-      <c r="S10" s="20">
-        <f t="shared" si="5"/>
-        <v>576</v>
-      </c>
       <c r="T10" s="27">
         <v>753</v>
       </c>
-      <c r="U10" s="9" t="s">
+      <c r="U10" s="27"/>
+      <c r="V10" s="27"/>
+      <c r="W10" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V10" s="9"/>
-      <c r="W10" s="20"/>
-      <c r="X10" s="20" t="str">
+      <c r="X10" s="9"/>
+      <c r="Y10" s="20"/>
+      <c r="Z10" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y10" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z10" s="10" t="s">
+      <c r="AA10" s="20" t="str">
+        <f>IF(OR(S10="",Z10=""),"",S10-Z10)</f>
+        <v/>
+      </c>
+      <c r="AB10" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="26.4">
+    <row r="11" spans="1:28" ht="25.5">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -4624,7 +4727,7 @@
         <v>320</v>
       </c>
       <c r="G11" s="18">
-        <f t="shared" ref="G11" si="6">ROUND(F11/0.8,0)</f>
+        <f t="shared" ref="G11" si="5">ROUND(F11/0.8,0)</f>
         <v>400</v>
       </c>
       <c r="H11" s="8" t="s">
@@ -4649,7 +4752,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P11" s="25" t="s">
@@ -4659,7 +4762,7 @@
         <v>2</v>
       </c>
       <c r="R11" s="24">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>288</v>
       </c>
       <c r="S11" s="20">
@@ -4669,24 +4772,26 @@
       <c r="T11" s="27">
         <v>801</v>
       </c>
-      <c r="U11" s="9" t="s">
+      <c r="U11" s="27"/>
+      <c r="V11" s="27"/>
+      <c r="W11" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V11" s="9"/>
-      <c r="W11" s="20"/>
-      <c r="X11" s="20" t="str">
-        <f t="shared" ref="X11" si="7">IF(OR(V11="",W11=""),"",V11*W11)</f>
-        <v/>
-      </c>
-      <c r="Y11" s="20" t="str">
-        <f t="shared" ref="Y11" si="8">IF(OR(S11="",X11=""),"",S11-X11)</f>
-        <v/>
-      </c>
-      <c r="Z11" s="10" t="s">
+      <c r="X11" s="9"/>
+      <c r="Y11" s="20"/>
+      <c r="Z11" s="20" t="str">
+        <f t="shared" ref="Z11" si="6">IF(OR(X11="",Y11=""),"",X11*Y11)</f>
+        <v/>
+      </c>
+      <c r="AA11" s="20" t="str">
+        <f>IF(OR(S11="",Z11=""),"",S11-Z11)</f>
+        <v/>
+      </c>
+      <c r="AB11" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="26.4">
+    <row r="12" spans="1:28" ht="25.5">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -4731,7 +4836,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P12" s="25" t="s">
@@ -4741,34 +4846,36 @@
         <v>6</v>
       </c>
       <c r="R12" s="24">
+        <f t="shared" si="3"/>
+        <v>864</v>
+      </c>
+      <c r="S12" s="20">
         <f t="shared" si="4"/>
         <v>864</v>
       </c>
-      <c r="S12" s="20">
-        <f t="shared" si="5"/>
-        <v>864</v>
-      </c>
       <c r="T12" s="27">
         <v>1107</v>
       </c>
-      <c r="U12" s="9" t="s">
+      <c r="U12" s="27"/>
+      <c r="V12" s="27"/>
+      <c r="W12" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V12" s="9"/>
-      <c r="W12" s="20"/>
-      <c r="X12" s="20" t="str">
+      <c r="X12" s="9"/>
+      <c r="Y12" s="20"/>
+      <c r="Z12" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y12" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z12" s="10" t="s">
+      <c r="AA12" s="20" t="str">
+        <f>IF(OR(S12="",Z12=""),"",S12-Z12)</f>
+        <v/>
+      </c>
+      <c r="AB12" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="26.4">
+    <row r="13" spans="1:28" ht="25.5">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -4813,7 +4920,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P13" s="25" t="s">
@@ -4823,34 +4930,36 @@
         <v>2</v>
       </c>
       <c r="R13" s="24">
+        <f t="shared" si="3"/>
+        <v>288</v>
+      </c>
+      <c r="S13" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
-      <c r="S13" s="20">
-        <f t="shared" si="5"/>
-        <v>288</v>
-      </c>
       <c r="T13" s="27">
         <v>740</v>
       </c>
-      <c r="U13" s="9" t="s">
+      <c r="U13" s="27"/>
+      <c r="V13" s="27"/>
+      <c r="W13" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V13" s="9"/>
-      <c r="W13" s="20"/>
-      <c r="X13" s="20" t="str">
+      <c r="X13" s="9"/>
+      <c r="Y13" s="20"/>
+      <c r="Z13" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y13" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z13" s="10" t="s">
+      <c r="AA13" s="20" t="str">
+        <f>IF(OR(S13="",Z13=""),"",S13-Z13)</f>
+        <v/>
+      </c>
+      <c r="AB13" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="26.4">
+    <row r="14" spans="1:28" ht="25.5">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -4895,7 +5004,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P14" s="25" t="s">
@@ -4905,34 +5014,36 @@
         <v>3</v>
       </c>
       <c r="R14" s="24">
+        <f t="shared" si="3"/>
+        <v>432</v>
+      </c>
+      <c r="S14" s="20">
         <f t="shared" si="4"/>
         <v>432</v>
       </c>
-      <c r="S14" s="20">
-        <f t="shared" si="5"/>
-        <v>432</v>
-      </c>
       <c r="T14" s="27">
         <v>865</v>
       </c>
-      <c r="U14" s="9" t="s">
+      <c r="U14" s="27"/>
+      <c r="V14" s="27"/>
+      <c r="W14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V14" s="9"/>
-      <c r="W14" s="20"/>
-      <c r="X14" s="20" t="str">
+      <c r="X14" s="9"/>
+      <c r="Y14" s="20"/>
+      <c r="Z14" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y14" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z14" s="10" t="s">
+      <c r="AA14" s="20" t="str">
+        <f>IF(OR(S14="",Z14=""),"",S14-Z14)</f>
+        <v/>
+      </c>
+      <c r="AB14" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="26.4">
+    <row r="15" spans="1:28" ht="25.5">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -4977,7 +5088,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P15" s="25" t="s">
@@ -4987,34 +5098,36 @@
         <v>2</v>
       </c>
       <c r="R15" s="24">
+        <f t="shared" si="3"/>
+        <v>288</v>
+      </c>
+      <c r="S15" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
-      <c r="S15" s="20">
-        <f t="shared" si="5"/>
-        <v>288</v>
-      </c>
       <c r="T15" s="27">
         <v>403</v>
       </c>
-      <c r="U15" s="9" t="s">
+      <c r="U15" s="27"/>
+      <c r="V15" s="27"/>
+      <c r="W15" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V15" s="9"/>
-      <c r="W15" s="20"/>
-      <c r="X15" s="20" t="str">
+      <c r="X15" s="9"/>
+      <c r="Y15" s="20"/>
+      <c r="Z15" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y15" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z15" s="10" t="s">
+      <c r="AA15" s="20" t="str">
+        <f>IF(OR(S15="",Z15=""),"",S15-Z15)</f>
+        <v/>
+      </c>
+      <c r="AB15" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="26.4">
+    <row r="16" spans="1:28" ht="25.5">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -5059,7 +5172,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P16" s="25" t="s">
@@ -5069,34 +5182,36 @@
         <v>1</v>
       </c>
       <c r="R16" s="24">
+        <f t="shared" si="3"/>
+        <v>144</v>
+      </c>
+      <c r="S16" s="20">
         <f t="shared" si="4"/>
         <v>144</v>
       </c>
-      <c r="S16" s="20">
-        <f t="shared" si="5"/>
-        <v>144</v>
-      </c>
       <c r="T16" s="27">
         <v>403</v>
       </c>
-      <c r="U16" s="9" t="s">
+      <c r="U16" s="27"/>
+      <c r="V16" s="27"/>
+      <c r="W16" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V16" s="9"/>
-      <c r="W16" s="20"/>
-      <c r="X16" s="20" t="str">
+      <c r="X16" s="9"/>
+      <c r="Y16" s="20"/>
+      <c r="Z16" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y16" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z16" s="10" t="s">
+      <c r="AA16" s="20" t="str">
+        <f>IF(OR(S16="",Z16=""),"",S16-Z16)</f>
+        <v/>
+      </c>
+      <c r="AB16" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:26" ht="26.4">
+    <row r="17" spans="1:28" ht="25.5">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -5141,7 +5256,7 @@
         <v>0</v>
       </c>
       <c r="O17" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P17" s="25" t="s">
@@ -5151,34 +5266,36 @@
         <v>4</v>
       </c>
       <c r="R17" s="24">
+        <f t="shared" si="3"/>
+        <v>576</v>
+      </c>
+      <c r="S17" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
-      <c r="S17" s="20">
-        <f t="shared" si="5"/>
-        <v>576</v>
-      </c>
       <c r="T17" s="27">
         <v>1069</v>
       </c>
-      <c r="U17" s="9" t="s">
+      <c r="U17" s="27"/>
+      <c r="V17" s="27"/>
+      <c r="W17" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V17" s="9"/>
-      <c r="W17" s="20"/>
-      <c r="X17" s="20" t="str">
+      <c r="X17" s="9"/>
+      <c r="Y17" s="20"/>
+      <c r="Z17" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y17" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z17" s="10" t="s">
+      <c r="AA17" s="20" t="str">
+        <f>IF(OR(S17="",Z17=""),"",S17-Z17)</f>
+        <v/>
+      </c>
+      <c r="AB17" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:26" ht="26.4">
+    <row r="18" spans="1:28" ht="25.5">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -5223,7 +5340,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P18" s="25" t="s">
@@ -5233,34 +5350,36 @@
         <v>2</v>
       </c>
       <c r="R18" s="24">
+        <f t="shared" si="3"/>
+        <v>288</v>
+      </c>
+      <c r="S18" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
-      <c r="S18" s="20">
-        <f t="shared" si="5"/>
-        <v>288</v>
-      </c>
       <c r="T18" s="27">
         <v>854</v>
       </c>
-      <c r="U18" s="9" t="s">
+      <c r="U18" s="27"/>
+      <c r="V18" s="27"/>
+      <c r="W18" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V18" s="9"/>
-      <c r="W18" s="20"/>
-      <c r="X18" s="20" t="str">
+      <c r="X18" s="9"/>
+      <c r="Y18" s="20"/>
+      <c r="Z18" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y18" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z18" s="10" t="s">
+      <c r="AA18" s="20" t="str">
+        <f>IF(OR(S18="",Z18=""),"",S18-Z18)</f>
+        <v/>
+      </c>
+      <c r="AB18" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:26" ht="26.4">
+    <row r="19" spans="1:28" ht="25.5">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -5305,7 +5424,7 @@
         <v>0</v>
       </c>
       <c r="O19" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P19" s="25" t="s">
@@ -5315,34 +5434,36 @@
         <v>6</v>
       </c>
       <c r="R19" s="24">
+        <f t="shared" si="3"/>
+        <v>864</v>
+      </c>
+      <c r="S19" s="20">
         <f t="shared" si="4"/>
         <v>864</v>
       </c>
-      <c r="S19" s="20">
-        <f t="shared" si="5"/>
-        <v>864</v>
-      </c>
       <c r="T19" s="27">
         <v>538</v>
       </c>
-      <c r="U19" s="9" t="s">
+      <c r="U19" s="27"/>
+      <c r="V19" s="27"/>
+      <c r="W19" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V19" s="9"/>
-      <c r="W19" s="20"/>
-      <c r="X19" s="20" t="str">
+      <c r="X19" s="9"/>
+      <c r="Y19" s="20"/>
+      <c r="Z19" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y19" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z19" s="10" t="s">
+      <c r="AA19" s="20" t="str">
+        <f>IF(OR(S19="",Z19=""),"",S19-Z19)</f>
+        <v/>
+      </c>
+      <c r="AB19" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:26" ht="26.4">
+    <row r="20" spans="1:28" ht="25.5">
       <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
@@ -5387,7 +5508,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P20" s="25" t="s">
@@ -5397,34 +5518,36 @@
         <v>4</v>
       </c>
       <c r="R20" s="24">
+        <f t="shared" si="3"/>
+        <v>576</v>
+      </c>
+      <c r="S20" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
-      <c r="S20" s="20">
-        <f t="shared" si="5"/>
-        <v>576</v>
-      </c>
       <c r="T20" s="27">
         <v>1064</v>
       </c>
-      <c r="U20" s="9" t="s">
+      <c r="U20" s="27"/>
+      <c r="V20" s="27"/>
+      <c r="W20" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V20" s="9"/>
-      <c r="W20" s="20"/>
-      <c r="X20" s="20" t="str">
+      <c r="X20" s="9"/>
+      <c r="Y20" s="20"/>
+      <c r="Z20" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y20" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z20" s="10" t="s">
+      <c r="AA20" s="20" t="str">
+        <f>IF(OR(S20="",Z20=""),"",S20-Z20)</f>
+        <v/>
+      </c>
+      <c r="AB20" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:26" ht="26.4">
+    <row r="21" spans="1:28" ht="25.5">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
@@ -5469,7 +5592,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P21" s="25" t="s">
@@ -5479,34 +5602,36 @@
         <v>1</v>
       </c>
       <c r="R21" s="24">
+        <f t="shared" si="3"/>
+        <v>144</v>
+      </c>
+      <c r="S21" s="20">
         <f t="shared" si="4"/>
         <v>144</v>
       </c>
-      <c r="S21" s="20">
-        <f t="shared" si="5"/>
-        <v>144</v>
-      </c>
       <c r="T21" s="27">
         <v>538</v>
       </c>
-      <c r="U21" s="9" t="s">
+      <c r="U21" s="27"/>
+      <c r="V21" s="27"/>
+      <c r="W21" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V21" s="9"/>
-      <c r="W21" s="20"/>
-      <c r="X21" s="20" t="str">
+      <c r="X21" s="9"/>
+      <c r="Y21" s="20"/>
+      <c r="Z21" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y21" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z21" s="10" t="s">
+      <c r="AA21" s="20" t="str">
+        <f>IF(OR(S21="",Z21=""),"",S21-Z21)</f>
+        <v/>
+      </c>
+      <c r="AB21" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:26" ht="26.4">
+    <row r="22" spans="1:28" ht="25.5">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
@@ -5551,7 +5676,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P22" s="25" t="s">
@@ -5561,34 +5686,36 @@
         <v>4</v>
       </c>
       <c r="R22" s="24">
+        <f t="shared" si="3"/>
+        <v>576</v>
+      </c>
+      <c r="S22" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
-      <c r="S22" s="20">
-        <f t="shared" si="5"/>
-        <v>576</v>
-      </c>
       <c r="T22" s="27">
         <v>1133</v>
       </c>
-      <c r="U22" s="9" t="s">
+      <c r="U22" s="27"/>
+      <c r="V22" s="27"/>
+      <c r="W22" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V22" s="9"/>
-      <c r="W22" s="20"/>
-      <c r="X22" s="20" t="str">
+      <c r="X22" s="9"/>
+      <c r="Y22" s="20"/>
+      <c r="Z22" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y22" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z22" s="10" t="s">
+      <c r="AA22" s="20" t="str">
+        <f>IF(OR(S22="",Z22=""),"",S22-Z22)</f>
+        <v/>
+      </c>
+      <c r="AB22" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:26" ht="26.4">
+    <row r="23" spans="1:28" ht="25.5">
       <c r="A23" s="6" t="s">
         <v>22</v>
       </c>
@@ -5633,7 +5760,7 @@
         <v>0</v>
       </c>
       <c r="O23" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P23" s="25" t="s">
@@ -5643,34 +5770,36 @@
         <v>2</v>
       </c>
       <c r="R23" s="24">
+        <f t="shared" si="3"/>
+        <v>288</v>
+      </c>
+      <c r="S23" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
-      <c r="S23" s="20">
-        <f t="shared" si="5"/>
-        <v>288</v>
-      </c>
       <c r="T23" s="27">
         <v>900</v>
       </c>
-      <c r="U23" s="9" t="s">
+      <c r="U23" s="27"/>
+      <c r="V23" s="27"/>
+      <c r="W23" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V23" s="9"/>
-      <c r="W23" s="20"/>
-      <c r="X23" s="20" t="str">
+      <c r="X23" s="9"/>
+      <c r="Y23" s="20"/>
+      <c r="Z23" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y23" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z23" s="10" t="s">
+      <c r="AA23" s="20" t="str">
+        <f>IF(OR(S23="",Z23=""),"",S23-Z23)</f>
+        <v/>
+      </c>
+      <c r="AB23" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:26" ht="26.4">
+    <row r="24" spans="1:28" ht="25.5">
       <c r="A24" s="6" t="s">
         <v>78</v>
       </c>
@@ -5725,7 +5854,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="24">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="S24" s="20">
@@ -5735,24 +5864,26 @@
       <c r="T24" s="29">
         <v>229</v>
       </c>
-      <c r="U24" s="9" t="s">
+      <c r="U24" s="29"/>
+      <c r="V24" s="29"/>
+      <c r="W24" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V24" s="9"/>
-      <c r="W24" s="20"/>
-      <c r="X24" s="20" t="str">
+      <c r="X24" s="9"/>
+      <c r="Y24" s="20"/>
+      <c r="Z24" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Y24" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Z24" s="10" t="s">
+      <c r="AA24" s="20" t="str">
+        <f>IF(OR(S24="",Z24=""),"",S24-Z24)</f>
+        <v/>
+      </c>
+      <c r="AB24" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="26.4">
+    <row r="25" spans="1:28" ht="25.5">
       <c r="A25" s="6" t="s">
         <v>78</v>
       </c>
@@ -5772,7 +5903,7 @@
         <v>40</v>
       </c>
       <c r="G25" s="18">
-        <f t="shared" ref="G25" si="9">ROUND(F25/0.8,0)</f>
+        <f t="shared" ref="G25" si="7">ROUND(F25/0.8,0)</f>
         <v>50</v>
       </c>
       <c r="H25" s="8" t="s">
@@ -5797,7 +5928,7 @@
         <v>2</v>
       </c>
       <c r="O25" s="20">
-        <f t="shared" ref="O25:O38" si="10">72*N25</f>
+        <f t="shared" ref="O25:O38" si="8">72*N25</f>
         <v>144</v>
       </c>
       <c r="P25" s="25" t="s">
@@ -5807,34 +5938,36 @@
         <v>0</v>
       </c>
       <c r="R25" s="24">
-        <f t="shared" ref="R25:R33" si="11">4*36*Q25</f>
+        <f t="shared" ref="R25:R33" si="9">4*36*Q25</f>
         <v>0</v>
       </c>
       <c r="S25" s="20">
-        <f t="shared" ref="S25:S38" si="12">O25</f>
+        <f t="shared" ref="S25:S38" si="10">O25</f>
         <v>144</v>
       </c>
       <c r="T25" s="29">
         <v>168</v>
       </c>
-      <c r="U25" s="9" t="s">
+      <c r="U25" s="29"/>
+      <c r="V25" s="29"/>
+      <c r="W25" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V25" s="9"/>
-      <c r="W25" s="20"/>
-      <c r="X25" s="20" t="str">
-        <f t="shared" ref="X25" si="13">IF(OR(V25="",W25=""),"",V25*W25)</f>
-        <v/>
-      </c>
-      <c r="Y25" s="20" t="str">
-        <f t="shared" ref="Y25" si="14">IF(OR(S25="",X25=""),"",S25-X25)</f>
-        <v/>
-      </c>
-      <c r="Z25" s="10" t="s">
+      <c r="X25" s="9"/>
+      <c r="Y25" s="20"/>
+      <c r="Z25" s="20" t="str">
+        <f t="shared" ref="Z25" si="11">IF(OR(X25="",Y25=""),"",X25*Y25)</f>
+        <v/>
+      </c>
+      <c r="AA25" s="20" t="str">
+        <f>IF(OR(S25="",Z25=""),"",S25-Z25)</f>
+        <v/>
+      </c>
+      <c r="AB25" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:26" ht="26.4">
+    <row r="26" spans="1:28" ht="25.5">
       <c r="A26" s="6" t="s">
         <v>78</v>
       </c>
@@ -5854,7 +5987,7 @@
         <v>80</v>
       </c>
       <c r="G26" s="18">
-        <f t="shared" ref="G26:G38" si="15">ROUND(F26/0.8,0)</f>
+        <f t="shared" ref="G26:G38" si="12">ROUND(F26/0.8,0)</f>
         <v>100</v>
       </c>
       <c r="H26" s="8" t="s">
@@ -5879,7 +6012,7 @@
         <v>0</v>
       </c>
       <c r="O26" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="P26" s="25" t="s">
@@ -5889,34 +6022,36 @@
         <v>0</v>
       </c>
       <c r="R26" s="24">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="S26" s="20">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="T26" s="29">
         <v>0</v>
       </c>
-      <c r="U26" s="9" t="s">
+      <c r="U26" s="29"/>
+      <c r="V26" s="29"/>
+      <c r="W26" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V26" s="9"/>
-      <c r="W26" s="20"/>
-      <c r="X26" s="20" t="str">
-        <f t="shared" ref="X26:X38" si="16">IF(OR(V26="",W26=""),"",V26*W26)</f>
-        <v/>
-      </c>
-      <c r="Y26" s="20" t="str">
-        <f t="shared" ref="Y26:Y38" si="17">IF(OR(S26="",X26=""),"",S26-X26)</f>
-        <v/>
-      </c>
-      <c r="Z26" s="10" t="s">
+      <c r="X26" s="9"/>
+      <c r="Y26" s="20"/>
+      <c r="Z26" s="20" t="str">
+        <f t="shared" ref="Z26:Z38" si="13">IF(OR(X26="",Y26=""),"",X26*Y26)</f>
+        <v/>
+      </c>
+      <c r="AA26" s="20" t="str">
+        <f>IF(OR(S26="",Z26=""),"",S26-Z26)</f>
+        <v/>
+      </c>
+      <c r="AB26" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:26" ht="26.4">
+    <row r="27" spans="1:28" ht="25.5">
       <c r="A27" s="6" t="s">
         <v>78</v>
       </c>
@@ -5936,7 +6071,7 @@
         <v>320</v>
       </c>
       <c r="G27" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H27" s="8" t="s">
@@ -5971,34 +6106,36 @@
         <v>0</v>
       </c>
       <c r="R27" s="24">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="S27" s="20">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>288</v>
       </c>
       <c r="T27" s="29">
         <v>291</v>
       </c>
-      <c r="U27" s="9" t="s">
+      <c r="U27" s="29"/>
+      <c r="V27" s="29"/>
+      <c r="W27" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V27" s="9"/>
-      <c r="W27" s="20"/>
-      <c r="X27" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y27" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z27" s="10" t="s">
+      <c r="X27" s="9"/>
+      <c r="Y27" s="20"/>
+      <c r="Z27" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA27" s="20" t="str">
+        <f>IF(OR(S27="",Z27=""),"",S27-Z27)</f>
+        <v/>
+      </c>
+      <c r="AB27" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:26" ht="26.4">
+    <row r="28" spans="1:28" ht="25.5">
       <c r="A28" s="6" t="s">
         <v>78</v>
       </c>
@@ -6018,7 +6155,7 @@
         <v>320</v>
       </c>
       <c r="G28" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H28" s="8" t="s">
@@ -6043,44 +6180,46 @@
         <v>4</v>
       </c>
       <c r="O28" s="20">
+        <f t="shared" si="8"/>
+        <v>288</v>
+      </c>
+      <c r="P28" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q28" s="24">
+        <v>0</v>
+      </c>
+      <c r="R28" s="24">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="S28" s="20">
         <f t="shared" si="10"/>
         <v>288</v>
       </c>
-      <c r="P28" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q28" s="24">
-        <v>0</v>
-      </c>
-      <c r="R28" s="24">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="S28" s="20">
-        <f t="shared" si="12"/>
-        <v>288</v>
-      </c>
       <c r="T28" s="29">
         <v>384</v>
       </c>
-      <c r="U28" s="9" t="s">
+      <c r="U28" s="29"/>
+      <c r="V28" s="29"/>
+      <c r="W28" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V28" s="9"/>
-      <c r="W28" s="20"/>
-      <c r="X28" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y28" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z28" s="10" t="s">
+      <c r="X28" s="9"/>
+      <c r="Y28" s="20"/>
+      <c r="Z28" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA28" s="20" t="str">
+        <f>IF(OR(S28="",Z28=""),"",S28-Z28)</f>
+        <v/>
+      </c>
+      <c r="AB28" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:26" ht="26.4">
+    <row r="29" spans="1:28" ht="25.5">
       <c r="A29" s="6" t="s">
         <v>78</v>
       </c>
@@ -6100,7 +6239,7 @@
         <v>320</v>
       </c>
       <c r="G29" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H29" s="8" t="s">
@@ -6125,44 +6264,46 @@
         <v>5</v>
       </c>
       <c r="O29" s="20">
+        <f t="shared" si="8"/>
+        <v>360</v>
+      </c>
+      <c r="P29" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q29" s="24">
+        <v>0</v>
+      </c>
+      <c r="R29" s="24">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="S29" s="20">
         <f t="shared" si="10"/>
         <v>360</v>
       </c>
-      <c r="P29" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q29" s="24">
-        <v>0</v>
-      </c>
-      <c r="R29" s="24">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="S29" s="20">
-        <f t="shared" si="12"/>
-        <v>360</v>
-      </c>
       <c r="T29" s="29">
         <v>375</v>
       </c>
-      <c r="U29" s="9" t="s">
+      <c r="U29" s="29"/>
+      <c r="V29" s="29"/>
+      <c r="W29" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V29" s="9"/>
-      <c r="W29" s="20"/>
-      <c r="X29" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y29" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z29" s="10" t="s">
+      <c r="X29" s="9"/>
+      <c r="Y29" s="20"/>
+      <c r="Z29" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA29" s="20" t="str">
+        <f>IF(OR(S29="",Z29=""),"",S29-Z29)</f>
+        <v/>
+      </c>
+      <c r="AB29" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:26" ht="26.4">
+    <row r="30" spans="1:28" ht="25.5">
       <c r="A30" s="6" t="s">
         <v>78</v>
       </c>
@@ -6182,7 +6323,7 @@
         <v>160</v>
       </c>
       <c r="G30" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>200</v>
       </c>
       <c r="H30" s="8" t="s">
@@ -6207,44 +6348,46 @@
         <v>7</v>
       </c>
       <c r="O30" s="20">
+        <f t="shared" si="8"/>
+        <v>504</v>
+      </c>
+      <c r="P30" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q30" s="24">
+        <v>0</v>
+      </c>
+      <c r="R30" s="24">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="S30" s="20">
         <f t="shared" si="10"/>
         <v>504</v>
       </c>
-      <c r="P30" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q30" s="24">
-        <v>0</v>
-      </c>
-      <c r="R30" s="24">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="S30" s="20">
-        <f t="shared" si="12"/>
-        <v>504</v>
-      </c>
       <c r="T30" s="29">
         <v>316</v>
       </c>
-      <c r="U30" s="9" t="s">
+      <c r="U30" s="29"/>
+      <c r="V30" s="29"/>
+      <c r="W30" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V30" s="9"/>
-      <c r="W30" s="20"/>
-      <c r="X30" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y30" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z30" s="10" t="s">
+      <c r="X30" s="9"/>
+      <c r="Y30" s="20"/>
+      <c r="Z30" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA30" s="20" t="str">
+        <f>IF(OR(S30="",Z30=""),"",S30-Z30)</f>
+        <v/>
+      </c>
+      <c r="AB30" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:26" ht="26.4">
+    <row r="31" spans="1:28" ht="25.5">
       <c r="A31" s="6" t="s">
         <v>78</v>
       </c>
@@ -6264,7 +6407,7 @@
         <v>320</v>
       </c>
       <c r="G31" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H31" s="8" t="s">
@@ -6289,44 +6432,46 @@
         <v>9</v>
       </c>
       <c r="O31" s="20">
+        <f t="shared" si="8"/>
+        <v>648</v>
+      </c>
+      <c r="P31" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q31" s="24">
+        <v>0</v>
+      </c>
+      <c r="R31" s="24">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="S31" s="20">
         <f t="shared" si="10"/>
         <v>648</v>
       </c>
-      <c r="P31" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q31" s="24">
-        <v>0</v>
-      </c>
-      <c r="R31" s="24">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="S31" s="20">
-        <f t="shared" si="12"/>
-        <v>648</v>
-      </c>
       <c r="T31" s="29">
         <v>476</v>
       </c>
-      <c r="U31" s="9" t="s">
+      <c r="U31" s="29"/>
+      <c r="V31" s="29"/>
+      <c r="W31" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V31" s="9"/>
-      <c r="W31" s="20"/>
-      <c r="X31" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y31" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z31" s="10" t="s">
+      <c r="X31" s="9"/>
+      <c r="Y31" s="20"/>
+      <c r="Z31" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA31" s="20" t="str">
+        <f>IF(OR(S31="",Z31=""),"",S31-Z31)</f>
+        <v/>
+      </c>
+      <c r="AB31" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:26" ht="26.4">
+    <row r="32" spans="1:28" ht="25.5">
       <c r="A32" s="6" t="s">
         <v>78</v>
       </c>
@@ -6346,7 +6491,7 @@
         <v>320</v>
       </c>
       <c r="G32" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H32" s="8" t="s">
@@ -6371,44 +6516,46 @@
         <v>6</v>
       </c>
       <c r="O32" s="20">
+        <f t="shared" si="8"/>
+        <v>432</v>
+      </c>
+      <c r="P32" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q32" s="24">
+        <v>0</v>
+      </c>
+      <c r="R32" s="24">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="S32" s="20">
         <f t="shared" si="10"/>
         <v>432</v>
       </c>
-      <c r="P32" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q32" s="24">
-        <v>0</v>
-      </c>
-      <c r="R32" s="24">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="S32" s="20">
-        <f t="shared" si="12"/>
-        <v>432</v>
-      </c>
       <c r="T32" s="29">
         <v>552</v>
       </c>
-      <c r="U32" s="9" t="s">
+      <c r="U32" s="29"/>
+      <c r="V32" s="29"/>
+      <c r="W32" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V32" s="9"/>
-      <c r="W32" s="20"/>
-      <c r="X32" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y32" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z32" s="10" t="s">
+      <c r="X32" s="9"/>
+      <c r="Y32" s="20"/>
+      <c r="Z32" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA32" s="20" t="str">
+        <f>IF(OR(S32="",Z32=""),"",S32-Z32)</f>
+        <v/>
+      </c>
+      <c r="AB32" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:26" ht="26.4">
+    <row r="33" spans="1:28" ht="25.5">
       <c r="A33" s="6" t="s">
         <v>78</v>
       </c>
@@ -6428,7 +6575,7 @@
         <v>80</v>
       </c>
       <c r="G33" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>100</v>
       </c>
       <c r="H33" s="8" t="s">
@@ -6453,44 +6600,46 @@
         <v>2</v>
       </c>
       <c r="O33" s="20">
+        <f t="shared" si="8"/>
+        <v>144</v>
+      </c>
+      <c r="P33" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q33" s="24">
+        <v>0</v>
+      </c>
+      <c r="R33" s="24">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="S33" s="20">
         <f t="shared" si="10"/>
         <v>144</v>
       </c>
-      <c r="P33" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q33" s="24">
-        <v>0</v>
-      </c>
-      <c r="R33" s="24">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="S33" s="20">
-        <f t="shared" si="12"/>
-        <v>144</v>
-      </c>
       <c r="T33" s="29">
         <v>227</v>
       </c>
-      <c r="U33" s="9" t="s">
+      <c r="U33" s="29"/>
+      <c r="V33" s="29"/>
+      <c r="W33" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V33" s="9"/>
-      <c r="W33" s="20"/>
-      <c r="X33" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y33" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z33" s="10" t="s">
+      <c r="X33" s="9"/>
+      <c r="Y33" s="20"/>
+      <c r="Z33" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA33" s="20" t="str">
+        <f>IF(OR(S33="",Z33=""),"",S33-Z33)</f>
+        <v/>
+      </c>
+      <c r="AB33" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:26" ht="26.4">
+    <row r="34" spans="1:28" ht="25.5">
       <c r="A34" s="6" t="s">
         <v>78</v>
       </c>
@@ -6510,7 +6659,7 @@
         <v>320</v>
       </c>
       <c r="G34" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H34" s="8" t="s">
@@ -6535,44 +6684,46 @@
         <v>9</v>
       </c>
       <c r="O34" s="20">
+        <f t="shared" si="8"/>
+        <v>648</v>
+      </c>
+      <c r="P34" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q34" s="24">
+        <v>0</v>
+      </c>
+      <c r="R34" s="24">
+        <f>4*36*Q34</f>
+        <v>0</v>
+      </c>
+      <c r="S34" s="20">
         <f t="shared" si="10"/>
         <v>648</v>
       </c>
-      <c r="P34" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q34" s="24">
-        <v>0</v>
-      </c>
-      <c r="R34" s="24">
-        <f>4*36*Q34</f>
-        <v>0</v>
-      </c>
-      <c r="S34" s="20">
-        <f t="shared" si="12"/>
-        <v>648</v>
-      </c>
       <c r="T34" s="29">
         <v>676</v>
       </c>
-      <c r="U34" s="9" t="s">
+      <c r="U34" s="29"/>
+      <c r="V34" s="29"/>
+      <c r="W34" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V34" s="9"/>
-      <c r="W34" s="20"/>
-      <c r="X34" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y34" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z34" s="10" t="s">
+      <c r="X34" s="9"/>
+      <c r="Y34" s="20"/>
+      <c r="Z34" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA34" s="20" t="str">
+        <f>IF(OR(S34="",Z34=""),"",S34-Z34)</f>
+        <v/>
+      </c>
+      <c r="AB34" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:26" ht="26.4">
+    <row r="35" spans="1:28" ht="25.5">
       <c r="A35" s="6" t="s">
         <v>78</v>
       </c>
@@ -6592,7 +6743,7 @@
         <v>80</v>
       </c>
       <c r="G35" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>100</v>
       </c>
       <c r="H35" s="8" t="s">
@@ -6627,7 +6778,7 @@
         <v>0</v>
       </c>
       <c r="R35" s="24">
-        <f t="shared" ref="R35:R38" si="18">4*36*Q35</f>
+        <f t="shared" ref="R35:R38" si="14">4*36*Q35</f>
         <v>0</v>
       </c>
       <c r="S35" s="20">
@@ -6637,24 +6788,26 @@
       <c r="T35" s="29">
         <v>273</v>
       </c>
-      <c r="U35" s="9" t="s">
+      <c r="U35" s="29"/>
+      <c r="V35" s="29"/>
+      <c r="W35" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V35" s="9"/>
-      <c r="W35" s="20"/>
-      <c r="X35" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y35" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z35" s="10" t="s">
+      <c r="X35" s="9"/>
+      <c r="Y35" s="20"/>
+      <c r="Z35" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA35" s="20" t="str">
+        <f>IF(OR(S35="",Z35=""),"",S35-Z35)</f>
+        <v/>
+      </c>
+      <c r="AB35" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="26.4">
+    <row r="36" spans="1:28" ht="25.5">
       <c r="A36" s="6" t="s">
         <v>78</v>
       </c>
@@ -6674,7 +6827,7 @@
         <v>320</v>
       </c>
       <c r="G36" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H36" s="8" t="s">
@@ -6699,44 +6852,46 @@
         <v>8</v>
       </c>
       <c r="O36" s="20">
+        <f t="shared" si="8"/>
+        <v>576</v>
+      </c>
+      <c r="P36" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q36" s="24">
+        <v>0</v>
+      </c>
+      <c r="R36" s="24">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="S36" s="20">
         <f t="shared" si="10"/>
         <v>576</v>
       </c>
-      <c r="P36" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q36" s="24">
-        <v>0</v>
-      </c>
-      <c r="R36" s="24">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="S36" s="20">
-        <f t="shared" si="12"/>
-        <v>576</v>
-      </c>
       <c r="T36" s="29">
         <v>622</v>
       </c>
-      <c r="U36" s="9" t="s">
+      <c r="U36" s="29"/>
+      <c r="V36" s="29"/>
+      <c r="W36" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="V36" s="9"/>
-      <c r="W36" s="20"/>
-      <c r="X36" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y36" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z36" s="10" t="s">
+      <c r="X36" s="9"/>
+      <c r="Y36" s="20"/>
+      <c r="Z36" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA36" s="20" t="str">
+        <f>IF(OR(S36="",Z36=""),"",S36-Z36)</f>
+        <v/>
+      </c>
+      <c r="AB36" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="37" spans="1:26" ht="26.4">
+    <row r="37" spans="1:28" ht="25.5">
       <c r="A37" s="6" t="s">
         <v>78</v>
       </c>
@@ -6756,7 +6911,7 @@
         <v>80</v>
       </c>
       <c r="G37" s="18">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>100</v>
       </c>
       <c r="H37" s="8" t="s">
@@ -6781,44 +6936,46 @@
         <v>1</v>
       </c>
       <c r="O37" s="20">
+        <f t="shared" si="8"/>
+        <v>72</v>
+      </c>
+      <c r="P37" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q37" s="24">
+        <v>0</v>
+      </c>
+      <c r="R37" s="24">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="S37" s="20">
         <f t="shared" si="10"/>
         <v>72</v>
       </c>
-      <c r="P37" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q37" s="24">
-        <v>0</v>
-      </c>
-      <c r="R37" s="24">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="S37" s="20">
-        <f t="shared" si="12"/>
-        <v>72</v>
-      </c>
       <c r="T37" s="29">
         <v>136</v>
       </c>
-      <c r="U37" s="9" t="s">
+      <c r="U37" s="29"/>
+      <c r="V37" s="29"/>
+      <c r="W37" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V37" s="9"/>
-      <c r="W37" s="20"/>
-      <c r="X37" s="20" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y37" s="20" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z37" s="10" t="s">
+      <c r="X37" s="9"/>
+      <c r="Y37" s="20"/>
+      <c r="Z37" s="20" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA37" s="20" t="str">
+        <f>IF(OR(S37="",Z37=""),"",S37-Z37)</f>
+        <v/>
+      </c>
+      <c r="AB37" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:26" ht="26.4">
+    <row r="38" spans="1:28" ht="25.5">
       <c r="A38" s="11" t="s">
         <v>78</v>
       </c>
@@ -6838,7 +6995,7 @@
         <v>320</v>
       </c>
       <c r="G38" s="19">
-        <f t="shared" si="15"/>
+        <f t="shared" si="12"/>
         <v>400</v>
       </c>
       <c r="H38" s="13" t="s">
@@ -6863,51 +7020,53 @@
         <v>8</v>
       </c>
       <c r="O38" s="20">
+        <f t="shared" si="8"/>
+        <v>576</v>
+      </c>
+      <c r="P38" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q38" s="24">
+        <v>0</v>
+      </c>
+      <c r="R38" s="24">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="S38" s="20">
         <f t="shared" si="10"/>
         <v>576</v>
       </c>
-      <c r="P38" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q38" s="24">
-        <v>0</v>
-      </c>
-      <c r="R38" s="24">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="S38" s="20">
-        <f t="shared" si="12"/>
-        <v>576</v>
-      </c>
       <c r="T38" s="29">
         <v>458</v>
       </c>
-      <c r="U38" s="14" t="s">
+      <c r="U38" s="29"/>
+      <c r="V38" s="29"/>
+      <c r="W38" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="V38" s="14"/>
-      <c r="W38" s="21"/>
-      <c r="X38" s="21" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="Y38" s="21" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="Z38" s="15" t="s">
+      <c r="X38" s="14"/>
+      <c r="Y38" s="21"/>
+      <c r="Z38" s="21" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="AA38" s="21" t="str">
+        <f>IF(OR(S38="",Z38=""),"",S38-Z38)</f>
+        <v/>
+      </c>
+      <c r="AB38" s="15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:26">
+    <row r="39" spans="1:28">
       <c r="M39" s="7"/>
       <c r="P39" s="7"/>
     </row>
-    <row r="40" spans="1:26">
+    <row r="40" spans="1:28">
       <c r="M40" s="7"/>
     </row>
-    <row r="41" spans="1:26">
+    <row r="41" spans="1:28">
       <c r="M41" s="7"/>
     </row>
   </sheetData>
@@ -6915,7 +7074,7 @@
     <mergeCell ref="A1:Z1"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="T4:T23">
+  <conditionalFormatting sqref="T4:V23 U25:V25">
     <cfRule type="expression" dxfId="3" priority="3">
       <formula>$T4&gt;=$F4</formula>
     </cfRule>
@@ -6939,7 +7098,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
@@ -6947,7 +7106,7 @@
     <col min="6" max="8" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21">
+    <row r="1" spans="1:8" ht="20.65">
       <c r="A1" s="36" t="s">
         <v>147</v>
       </c>
@@ -6959,7 +7118,7 @@
       <c r="G1" s="36"/>
       <c r="H1" s="36"/>
     </row>
-    <row r="2" spans="1:8" ht="27.6">
+    <row r="2" spans="1:8" ht="27.75">
       <c r="A2" s="1" t="s">
         <v>148</v>
       </c>
@@ -6985,7 +7144,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="27.6">
+    <row r="3" spans="1:8" ht="27">
       <c r="A3" s="2" t="s">
         <v>69</v>
       </c>
@@ -7012,7 +7171,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="27.6">
+    <row r="4" spans="1:8" ht="27">
       <c r="A4" s="2" t="s">
         <v>158</v>
       </c>
@@ -7174,7 +7333,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="27.6">
+    <row r="10" spans="1:8" ht="27">
       <c r="A10" s="2" t="s">
         <v>174</v>
       </c>

</xml_diff>

<commit_message>
Building B ground floor, ugr and uniformity
</commit_message>
<xml_diff>
--- a/excel/Building A B and carpark Lighting New.xlsx
+++ b/excel/Building A B and carpark Lighting New.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lsen906\Documents\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F835CACE-7537-4F06-AA1F-FE3CCD4C11F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8851FCBE-8EC6-40CC-9AA9-420AB01ADE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -28,15 +28,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="202">
   <si>
     <t>Building A — Lighting Place Schedule</t>
   </si>
@@ -633,12 +630,24 @@
   </si>
   <si>
     <t>Glare (UGGR)</t>
+  </si>
+  <si>
+    <t>Slope: 0.00 Flat: 0.87</t>
+  </si>
+  <si>
+    <t>25 Slope: 18.5 Flat: 10.2</t>
+  </si>
+  <si>
+    <t>WC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -679,7 +688,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -735,7 +744,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -820,7 +835,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -919,14 +934,26 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="9" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -937,7 +964,35 @@
     <cellStyle name="Normal 5" xfId="4" xr:uid="{ED6D2035-F9DA-4B1D-B2ED-B5DB87628F59}"/>
     <cellStyle name="Normal 6" xfId="5" xr:uid="{FCC80704-4661-421C-AAE8-B6CB6410940C}"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1148,7 +1203,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB36"/>
-  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -1161,40 +1216,40 @@
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="8.3125" customWidth="1"/>
+    <col min="17" max="17" width="8.375" customWidth="1"/>
     <col min="18" max="20" width="12" customWidth="1"/>
     <col min="21" max="22" width="14" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="20.65">
-      <c r="A1" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-    </row>
-    <row r="2" spans="1:28" ht="41.65">
+    <row r="1" spans="1:28" ht="20.25">
+      <c r="A1" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="34"/>
+      <c r="P1" s="34"/>
+      <c r="Q1" s="34"/>
+      <c r="R1" s="34"/>
+      <c r="S1" s="34"/>
+      <c r="T1" s="34"/>
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
+    </row>
+    <row r="2" spans="1:28" ht="45">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1280,7 +1335,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="27">
+    <row r="3" spans="1:28" ht="28.5">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -1349,14 +1404,14 @@
         <v/>
       </c>
       <c r="AA3" s="20" t="str">
-        <f>IF(OR(S3="",Z3=""),"",S3-Z3)</f>
+        <f t="shared" ref="AA3:AA36" si="1">IF(OR(S3="",Z3=""),"",S3-Z3)</f>
         <v/>
       </c>
       <c r="AB3" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="27">
+    <row r="4" spans="1:28" ht="28.5">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -1432,7 +1487,7 @@
         <v/>
       </c>
       <c r="AA4" s="20" t="str">
-        <f>IF(OR(S4="",Z4=""),"",S4-Z4)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB4" s="10" t="s">
@@ -1490,7 +1545,7 @@
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
       <c r="S5" s="20">
-        <f t="shared" ref="S5:S35" si="1">IF(OR(N5="",O5=""),"",N5*O5)</f>
+        <f t="shared" ref="S5:S35" si="2">IF(OR(N5="",O5=""),"",N5*O5)</f>
         <v>72</v>
       </c>
       <c r="T5" s="27">
@@ -1504,11 +1559,11 @@
       <c r="X5" s="9"/>
       <c r="Y5" s="20"/>
       <c r="Z5" s="20" t="str">
-        <f t="shared" ref="Z5:Z36" si="2">IF(OR(X5="",Y5=""),"",X5*Y5)</f>
+        <f t="shared" ref="Z5:Z36" si="3">IF(OR(X5="",Y5=""),"",X5*Y5)</f>
         <v/>
       </c>
       <c r="AA5" s="20" t="str">
-        <f>IF(OR(S5="",Z5=""),"",S5-Z5)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB5" s="10" t="s">
@@ -1566,7 +1621,7 @@
       <c r="Q6" s="24"/>
       <c r="R6" s="24"/>
       <c r="S6" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T6" s="27">
@@ -1580,11 +1635,11 @@
       <c r="X6" s="9"/>
       <c r="Y6" s="20"/>
       <c r="Z6" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA6" s="20" t="str">
-        <f>IF(OR(S6="",Z6=""),"",S6-Z6)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB6" s="10" t="s">
@@ -1642,7 +1697,7 @@
       <c r="Q7" s="24"/>
       <c r="R7" s="24"/>
       <c r="S7" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T7" s="27">
@@ -1656,11 +1711,11 @@
       <c r="X7" s="9"/>
       <c r="Y7" s="20"/>
       <c r="Z7" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA7" s="20" t="str">
-        <f>IF(OR(S7="",Z7=""),"",S7-Z7)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB7" s="10" t="s">
@@ -1718,7 +1773,7 @@
       <c r="Q8" s="24"/>
       <c r="R8" s="24"/>
       <c r="S8" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T8" s="27">
@@ -1732,11 +1787,11 @@
       <c r="X8" s="9"/>
       <c r="Y8" s="20"/>
       <c r="Z8" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA8" s="20" t="str">
-        <f>IF(OR(S8="",Z8=""),"",S8-Z8)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB8" s="10" t="s">
@@ -1794,7 +1849,7 @@
       <c r="Q9" s="24"/>
       <c r="R9" s="24"/>
       <c r="S9" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T9" s="27">
@@ -1808,18 +1863,18 @@
       <c r="X9" s="9"/>
       <c r="Y9" s="20"/>
       <c r="Z9" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA9" s="20" t="str">
-        <f>IF(OR(S9="",Z9=""),"",S9-Z9)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB9" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="27">
+    <row r="10" spans="1:28" ht="28.5">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1891,11 +1946,11 @@
       <c r="X10" s="9"/>
       <c r="Y10" s="20"/>
       <c r="Z10" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA10" s="20" t="str">
-        <f>IF(OR(S10="",Z10=""),"",S10-Z10)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB10" s="10" t="s">
@@ -1953,7 +2008,7 @@
       <c r="Q11" s="24"/>
       <c r="R11" s="24"/>
       <c r="S11" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T11" s="27">
@@ -1970,7 +2025,7 @@
         <v/>
       </c>
       <c r="AA11" s="20" t="str">
-        <f>IF(OR(S11="",Z11=""),"",S11-Z11)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB11" s="10" t="s">
@@ -2028,7 +2083,7 @@
       <c r="Q12" s="24"/>
       <c r="R12" s="24"/>
       <c r="S12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T12" s="27">
@@ -2046,7 +2101,7 @@
         <v>#REF!</v>
       </c>
       <c r="AA12" s="20" t="e">
-        <f>IF(OR(S12="",Z12=""),"",S12-Z12)</f>
+        <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
       <c r="AB12" s="10" t="s">
@@ -2104,7 +2159,7 @@
       <c r="Q13" s="24"/>
       <c r="R13" s="24"/>
       <c r="S13" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T13" s="27">
@@ -2118,11 +2173,11 @@
       <c r="X13" s="9"/>
       <c r="Y13" s="20"/>
       <c r="Z13" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA13" s="20" t="str">
-        <f>IF(OR(S13="",Z13=""),"",S13-Z13)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB13" s="10" t="s">
@@ -2180,7 +2235,7 @@
       <c r="Q14" s="24"/>
       <c r="R14" s="24"/>
       <c r="S14" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>864</v>
       </c>
       <c r="T14" s="27">
@@ -2194,11 +2249,11 @@
       <c r="X14" s="9"/>
       <c r="Y14" s="20"/>
       <c r="Z14" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA14" s="20" t="str">
-        <f>IF(OR(S14="",Z14=""),"",S14-Z14)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB14" s="10" t="s">
@@ -2256,7 +2311,7 @@
       <c r="Q15" s="24"/>
       <c r="R15" s="24"/>
       <c r="S15" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="T15" s="27">
@@ -2270,11 +2325,11 @@
       <c r="X15" s="9"/>
       <c r="Y15" s="20"/>
       <c r="Z15" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA15" s="20" t="str">
-        <f>IF(OR(S15="",Z15=""),"",S15-Z15)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB15" s="10" t="s">
@@ -2332,7 +2387,7 @@
       <c r="Q16" s="24"/>
       <c r="R16" s="24"/>
       <c r="S16" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="T16" s="27">
@@ -2346,18 +2401,18 @@
       <c r="X16" s="9"/>
       <c r="Y16" s="20"/>
       <c r="Z16" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA16" s="20" t="str">
-        <f>IF(OR(S16="",Z16=""),"",S16-Z16)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB16" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="27">
+    <row r="17" spans="1:28" ht="28.5">
       <c r="A17" s="6" t="s">
         <v>78</v>
       </c>
@@ -2408,7 +2463,7 @@
       <c r="Q17" s="24"/>
       <c r="R17" s="24"/>
       <c r="S17" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T17" s="27">
@@ -2422,18 +2477,18 @@
       <c r="X17" s="9"/>
       <c r="Y17" s="20"/>
       <c r="Z17" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA17" s="20" t="str">
-        <f>IF(OR(S17="",Z17=""),"",S17-Z17)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB17" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="27">
+    <row r="18" spans="1:28" ht="28.5">
       <c r="A18" s="6" t="s">
         <v>78</v>
       </c>
@@ -2484,7 +2539,7 @@
       <c r="Q18" s="24"/>
       <c r="R18" s="24"/>
       <c r="S18" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T18" s="27">
@@ -2498,11 +2553,11 @@
       <c r="X18" s="9"/>
       <c r="Y18" s="20"/>
       <c r="Z18" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA18" s="20" t="str">
-        <f>IF(OR(S18="",Z18=""),"",S18-Z18)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB18" s="10" t="s">
@@ -2560,7 +2615,7 @@
       <c r="Q19" s="24"/>
       <c r="R19" s="24"/>
       <c r="S19" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="T19" s="27">
@@ -2574,11 +2629,11 @@
       <c r="X19" s="9"/>
       <c r="Y19" s="20"/>
       <c r="Z19" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA19" s="20" t="str">
-        <f>IF(OR(S19="",Z19=""),"",S19-Z19)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB19" s="10" t="s">
@@ -2636,7 +2691,7 @@
       <c r="Q20" s="24"/>
       <c r="R20" s="24"/>
       <c r="S20" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1008</v>
       </c>
       <c r="T20" s="27">
@@ -2650,18 +2705,18 @@
       <c r="X20" s="9"/>
       <c r="Y20" s="20"/>
       <c r="Z20" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA20" s="20" t="str">
-        <f>IF(OR(S20="",Z20=""),"",S20-Z20)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB20" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="27">
+    <row r="21" spans="1:28" ht="28.5">
       <c r="A21" s="6" t="s">
         <v>78</v>
       </c>
@@ -2712,7 +2767,7 @@
       <c r="Q21" s="24"/>
       <c r="R21" s="24"/>
       <c r="S21" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T21" s="27">
@@ -2726,11 +2781,11 @@
       <c r="X21" s="9"/>
       <c r="Y21" s="20"/>
       <c r="Z21" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA21" s="20" t="str">
-        <f>IF(OR(S21="",Z21=""),"",S21-Z21)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB21" s="10" t="s">
@@ -2788,7 +2843,7 @@
       <c r="Q22" s="24"/>
       <c r="R22" s="24"/>
       <c r="S22" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>144</v>
       </c>
       <c r="T22" s="27">
@@ -2802,11 +2857,11 @@
       <c r="X22" s="9"/>
       <c r="Y22" s="20"/>
       <c r="Z22" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA22" s="20" t="str">
-        <f>IF(OR(S22="",Z22=""),"",S22-Z22)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB22" s="10" t="s">
@@ -2864,7 +2919,7 @@
       <c r="Q23" s="24"/>
       <c r="R23" s="24"/>
       <c r="S23" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>864</v>
       </c>
       <c r="T23" s="27">
@@ -2878,11 +2933,11 @@
       <c r="X23" s="9"/>
       <c r="Y23" s="20"/>
       <c r="Z23" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA23" s="20" t="str">
-        <f>IF(OR(S23="",Z23=""),"",S23-Z23)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB23" s="10" t="s">
@@ -2940,7 +2995,7 @@
       <c r="Q24" s="24"/>
       <c r="R24" s="24"/>
       <c r="S24" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T24" s="27">
@@ -2954,11 +3009,11 @@
       <c r="X24" s="9"/>
       <c r="Y24" s="20"/>
       <c r="Z24" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA24" s="20" t="str">
-        <f>IF(OR(S24="",Z24=""),"",S24-Z24)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB24" s="10" t="s">
@@ -3016,7 +3071,7 @@
       <c r="Q25" s="24"/>
       <c r="R25" s="24"/>
       <c r="S25" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T25" s="27">
@@ -3030,11 +3085,11 @@
       <c r="X25" s="9"/>
       <c r="Y25" s="20"/>
       <c r="Z25" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA25" s="20" t="str">
-        <f>IF(OR(S25="",Z25=""),"",S25-Z25)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB25" s="10" t="s">
@@ -3092,7 +3147,7 @@
       <c r="Q26" s="24"/>
       <c r="R26" s="24"/>
       <c r="S26" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1152</v>
       </c>
       <c r="T26" s="27">
@@ -3106,18 +3161,18 @@
       <c r="X26" s="9"/>
       <c r="Y26" s="20"/>
       <c r="Z26" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA26" s="20" t="str">
-        <f>IF(OR(S26="",Z26=""),"",S26-Z26)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB26" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="27">
+    <row r="27" spans="1:28" ht="28.5">
       <c r="A27" s="6" t="s">
         <v>78</v>
       </c>
@@ -3168,7 +3223,7 @@
       <c r="Q27" s="24"/>
       <c r="R27" s="24"/>
       <c r="S27" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T27" s="27">
@@ -3182,11 +3237,11 @@
       <c r="X27" s="9"/>
       <c r="Y27" s="20"/>
       <c r="Z27" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA27" s="20" t="str">
-        <f>IF(OR(S27="",Z27=""),"",S27-Z27)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB27" s="10" t="s">
@@ -3244,7 +3299,7 @@
       <c r="Q28" s="24"/>
       <c r="R28" s="24"/>
       <c r="S28" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1152</v>
       </c>
       <c r="T28" s="27">
@@ -3258,18 +3313,18 @@
       <c r="X28" s="9"/>
       <c r="Y28" s="20"/>
       <c r="Z28" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA28" s="20" t="str">
-        <f>IF(OR(S28="",Z28=""),"",S28-Z28)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB28" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="27">
+    <row r="29" spans="1:28" ht="28.5">
       <c r="A29" s="6" t="s">
         <v>78</v>
       </c>
@@ -3320,7 +3375,7 @@
       <c r="Q29" s="24"/>
       <c r="R29" s="24"/>
       <c r="S29" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T29" s="27">
@@ -3334,11 +3389,11 @@
       <c r="X29" s="9"/>
       <c r="Y29" s="20"/>
       <c r="Z29" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA29" s="20" t="str">
-        <f>IF(OR(S29="",Z29=""),"",S29-Z29)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB29" s="10" t="s">
@@ -3396,7 +3451,7 @@
       <c r="Q30" s="24"/>
       <c r="R30" s="24"/>
       <c r="S30" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T30" s="27">
@@ -3410,11 +3465,11 @@
       <c r="X30" s="9"/>
       <c r="Y30" s="20"/>
       <c r="Z30" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA30" s="20" t="str">
-        <f>IF(OR(S30="",Z30=""),"",S30-Z30)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB30" s="10" t="s">
@@ -3472,7 +3527,7 @@
       <c r="Q31" s="24"/>
       <c r="R31" s="24"/>
       <c r="S31" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T31" s="27">
@@ -3486,11 +3541,11 @@
       <c r="X31" s="9"/>
       <c r="Y31" s="20"/>
       <c r="Z31" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA31" s="20" t="str">
-        <f>IF(OR(S31="",Z31=""),"",S31-Z31)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB31" s="10" t="s">
@@ -3548,7 +3603,7 @@
       <c r="Q32" s="24"/>
       <c r="R32" s="24"/>
       <c r="S32" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="T32" s="27">
@@ -3562,11 +3617,11 @@
       <c r="X32" s="9"/>
       <c r="Y32" s="20"/>
       <c r="Z32" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA32" s="20" t="str">
-        <f>IF(OR(S32="",Z32=""),"",S32-Z32)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB32" s="10" t="s">
@@ -3624,7 +3679,7 @@
       <c r="Q33" s="24"/>
       <c r="R33" s="24"/>
       <c r="S33" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T33" s="27">
@@ -3638,11 +3693,11 @@
       <c r="X33" s="9"/>
       <c r="Y33" s="20"/>
       <c r="Z33" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA33" s="20" t="str">
-        <f>IF(OR(S33="",Z33=""),"",S33-Z33)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB33" s="10" t="s">
@@ -3700,7 +3755,7 @@
       <c r="Q34" s="24"/>
       <c r="R34" s="24"/>
       <c r="S34" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="T34" s="27">
@@ -3714,11 +3769,11 @@
       <c r="X34" s="9"/>
       <c r="Y34" s="20"/>
       <c r="Z34" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA34" s="20" t="str">
-        <f>IF(OR(S34="",Z34=""),"",S34-Z34)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB34" s="10" t="s">
@@ -3776,7 +3831,7 @@
       <c r="Q35" s="24"/>
       <c r="R35" s="24"/>
       <c r="S35" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="T35" s="27">
@@ -3790,11 +3845,11 @@
       <c r="X35" s="9"/>
       <c r="Y35" s="20"/>
       <c r="Z35" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA35" s="20" t="str">
-        <f>IF(OR(S35="",Z35=""),"",S35-Z35)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB35" s="10" t="s">
@@ -3866,11 +3921,11 @@
       <c r="X36" s="14"/>
       <c r="Y36" s="21"/>
       <c r="Z36" s="21" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AA36" s="21" t="str">
-        <f>IF(OR(S36="",Z36=""),"",S36-Z36)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="AB36" s="15" t="s">
@@ -3882,10 +3937,10 @@
     <mergeCell ref="A1:W1"/>
   </mergeCells>
   <conditionalFormatting sqref="T4:V36">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>$T4&lt;$F4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>$T4&gt;=$F4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3897,59 +3952,63 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AB41"/>
-  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="7" width="14" customWidth="1"/>
-    <col min="8" max="9" width="18" customWidth="1"/>
+    <col min="8" max="8" width="16.875" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="34" customWidth="1"/>
     <col min="11" max="11" width="30" customWidth="1"/>
     <col min="12" max="12" width="34" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="15" width="12" customWidth="1"/>
+    <col min="13" max="13" width="17.25" customWidth="1"/>
+    <col min="14" max="14" width="11.75" customWidth="1"/>
+    <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="15.6875" customWidth="1"/>
+    <col min="17" max="17" width="15.75" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="24" customWidth="1"/>
+    <col min="21" max="21" width="19" customWidth="1"/>
     <col min="22" max="23" width="12" customWidth="1"/>
     <col min="24" max="25" width="14" customWidth="1"/>
     <col min="26" max="26" width="16" customWidth="1"/>
+    <col min="27" max="27" width="12.375" customWidth="1"/>
+    <col min="28" max="28" width="14.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="20.65">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:28" ht="20.25">
+      <c r="A1" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="35"/>
-      <c r="Y1" s="35"/>
-      <c r="Z1" s="35"/>
-    </row>
-    <row r="2" spans="1:28" ht="41.65">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="34"/>
+      <c r="P1" s="34"/>
+      <c r="Q1" s="34"/>
+      <c r="R1" s="34"/>
+      <c r="S1" s="34"/>
+      <c r="T1" s="34"/>
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
+      <c r="X1" s="34"/>
+      <c r="Y1" s="34"/>
+      <c r="Z1" s="34"/>
+    </row>
+    <row r="2" spans="1:28" ht="45">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -4100,8 +4159,12 @@
       <c r="T3" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="U3" s="27"/>
-      <c r="V3" s="27"/>
+      <c r="U3" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="V3" s="38" t="s">
+        <v>200</v>
+      </c>
       <c r="W3" s="9" t="s">
         <v>30</v>
       </c>
@@ -4112,7 +4175,7 @@
         <v/>
       </c>
       <c r="AA3" s="20" t="str">
-        <f>IF(OR(S3="",Z3=""),"",S3-Z3)</f>
+        <f t="shared" ref="AA3:AA38" si="2">IF(OR(S3="",Z3=""),"",S3-Z3)</f>
         <v/>
       </c>
       <c r="AB3" s="10" t="s">
@@ -4164,7 +4227,7 @@
         <v>2</v>
       </c>
       <c r="O4" s="20">
-        <f t="shared" ref="O4:O23" si="2">2*36*N4</f>
+        <f t="shared" ref="O4:O23" si="3">2*36*N4</f>
         <v>144</v>
       </c>
       <c r="P4" s="25" t="s">
@@ -4174,18 +4237,22 @@
         <v>5</v>
       </c>
       <c r="R4" s="24">
-        <f t="shared" ref="R4:R24" si="3">4*36*Q4</f>
+        <f t="shared" ref="R4:R24" si="4">4*36*Q4</f>
         <v>720</v>
       </c>
       <c r="S4" s="20">
-        <f t="shared" ref="S4:S23" si="4">O4+R4</f>
+        <f t="shared" ref="S4:S23" si="5">O4+R4</f>
         <v>864</v>
       </c>
       <c r="T4" s="27">
         <v>380</v>
       </c>
-      <c r="U4" s="27"/>
-      <c r="V4" s="27"/>
+      <c r="U4" s="39">
+        <v>0.25</v>
+      </c>
+      <c r="V4" s="38">
+        <v>29</v>
+      </c>
       <c r="W4" s="9" t="s">
         <v>30</v>
       </c>
@@ -4196,7 +4263,7 @@
         <v/>
       </c>
       <c r="AA4" s="20" t="str">
-        <f>IF(OR(S4="",Z4=""),"",S4-Z4)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB4" s="10" t="s">
@@ -4248,7 +4315,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P5" s="25" t="s">
@@ -4258,18 +4325,22 @@
         <v>1</v>
       </c>
       <c r="R5" s="24">
-        <f t="shared" si="3"/>
-        <v>144</v>
-      </c>
-      <c r="S5" s="20">
         <f t="shared" si="4"/>
         <v>144</v>
       </c>
+      <c r="S5" s="20">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
       <c r="T5" s="27">
         <v>325</v>
       </c>
-      <c r="U5" s="27"/>
-      <c r="V5" s="27"/>
+      <c r="U5" s="37">
+        <v>0.49</v>
+      </c>
+      <c r="V5" s="29">
+        <v>18</v>
+      </c>
       <c r="W5" s="9" t="s">
         <v>30</v>
       </c>
@@ -4280,7 +4351,7 @@
         <v/>
       </c>
       <c r="AA5" s="20" t="str">
-        <f>IF(OR(S5="",Z5=""),"",S5-Z5)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB5" s="10" t="s">
@@ -4332,7 +4403,7 @@
         <v>1</v>
       </c>
       <c r="O6" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P6" s="25" t="s">
@@ -4342,18 +4413,22 @@
         <v>0</v>
       </c>
       <c r="R6" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S6" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T6" s="27">
         <v>205</v>
       </c>
-      <c r="U6" s="27"/>
-      <c r="V6" s="27"/>
+      <c r="U6" s="37">
+        <v>0.9</v>
+      </c>
+      <c r="V6" s="29">
+        <v>21</v>
+      </c>
       <c r="W6" s="9" t="s">
         <v>30</v>
       </c>
@@ -4364,7 +4439,7 @@
         <v/>
       </c>
       <c r="AA6" s="20" t="str">
-        <f>IF(OR(S6="",Z6=""),"",S6-Z6)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB6" s="10" t="s">
@@ -4379,7 +4454,7 @@
         <v>46</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>39</v>
+        <v>201</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>40</v>
@@ -4416,7 +4491,7 @@
         <v>1</v>
       </c>
       <c r="O7" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P7" s="25" t="s">
@@ -4426,18 +4501,22 @@
         <v>0</v>
       </c>
       <c r="R7" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S7" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T7" s="27">
         <v>201</v>
       </c>
-      <c r="U7" s="27"/>
-      <c r="V7" s="27"/>
+      <c r="U7" s="37">
+        <v>0.66</v>
+      </c>
+      <c r="V7" s="29">
+        <v>21</v>
+      </c>
       <c r="W7" s="9" t="s">
         <v>30</v>
       </c>
@@ -4448,7 +4527,7 @@
         <v/>
       </c>
       <c r="AA7" s="20" t="str">
-        <f>IF(OR(S7="",Z7=""),"",S7-Z7)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB7" s="10" t="s">
@@ -4463,7 +4542,7 @@
         <v>49</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>39</v>
+        <v>201</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>40</v>
@@ -4500,7 +4579,7 @@
         <v>1</v>
       </c>
       <c r="O8" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P8" s="25" t="s">
@@ -4510,18 +4589,22 @@
         <v>0</v>
       </c>
       <c r="R8" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S8" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T8" s="27">
         <v>186</v>
       </c>
-      <c r="U8" s="27"/>
-      <c r="V8" s="27"/>
+      <c r="U8" s="37">
+        <v>0.82</v>
+      </c>
+      <c r="V8" s="29">
+        <v>21</v>
+      </c>
       <c r="W8" s="9" t="s">
         <v>30</v>
       </c>
@@ -4532,7 +4615,7 @@
         <v/>
       </c>
       <c r="AA8" s="20" t="str">
-        <f>IF(OR(S8="",Z8=""),"",S8-Z8)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB8" s="10" t="s">
@@ -4584,7 +4667,7 @@
         <v>1</v>
       </c>
       <c r="O9" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="P9" s="25" t="s">
@@ -4594,18 +4677,22 @@
         <v>0</v>
       </c>
       <c r="R9" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S9" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="T9" s="27">
         <v>187</v>
       </c>
-      <c r="U9" s="27"/>
-      <c r="V9" s="27"/>
+      <c r="U9" s="37">
+        <v>0.83</v>
+      </c>
+      <c r="V9" s="29">
+        <v>21</v>
+      </c>
       <c r="W9" s="9" t="s">
         <v>30</v>
       </c>
@@ -4616,7 +4703,7 @@
         <v/>
       </c>
       <c r="AA9" s="20" t="str">
-        <f>IF(OR(S9="",Z9=""),"",S9-Z9)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB9" s="10" t="s">
@@ -4668,7 +4755,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P10" s="25" t="s">
@@ -4678,18 +4765,22 @@
         <v>4</v>
       </c>
       <c r="R10" s="24">
-        <f t="shared" si="3"/>
-        <v>576</v>
-      </c>
-      <c r="S10" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
+      <c r="S10" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
       <c r="T10" s="27">
         <v>753</v>
       </c>
-      <c r="U10" s="27"/>
-      <c r="V10" s="27"/>
+      <c r="U10" s="39">
+        <v>0.43</v>
+      </c>
+      <c r="V10" s="29">
+        <v>19</v>
+      </c>
       <c r="W10" s="9" t="s">
         <v>56</v>
       </c>
@@ -4700,7 +4791,7 @@
         <v/>
       </c>
       <c r="AA10" s="20" t="str">
-        <f>IF(OR(S10="",Z10=""),"",S10-Z10)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB10" s="10" t="s">
@@ -4727,7 +4818,7 @@
         <v>320</v>
       </c>
       <c r="G11" s="18">
-        <f t="shared" ref="G11" si="5">ROUND(F11/0.8,0)</f>
+        <f t="shared" ref="G11" si="6">ROUND(F11/0.8,0)</f>
         <v>400</v>
       </c>
       <c r="H11" s="8" t="s">
@@ -4752,7 +4843,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P11" s="25" t="s">
@@ -4762,7 +4853,7 @@
         <v>2</v>
       </c>
       <c r="R11" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>288</v>
       </c>
       <c r="S11" s="20">
@@ -4772,19 +4863,23 @@
       <c r="T11" s="27">
         <v>801</v>
       </c>
-      <c r="U11" s="27"/>
-      <c r="V11" s="27"/>
+      <c r="U11" s="39">
+        <v>0.53</v>
+      </c>
+      <c r="V11" s="29">
+        <v>18</v>
+      </c>
       <c r="W11" s="9" t="s">
         <v>56</v>
       </c>
       <c r="X11" s="9"/>
       <c r="Y11" s="20"/>
       <c r="Z11" s="20" t="str">
-        <f t="shared" ref="Z11" si="6">IF(OR(X11="",Y11=""),"",X11*Y11)</f>
+        <f t="shared" ref="Z11" si="7">IF(OR(X11="",Y11=""),"",X11*Y11)</f>
         <v/>
       </c>
       <c r="AA11" s="20" t="str">
-        <f>IF(OR(S11="",Z11=""),"",S11-Z11)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB11" s="10" t="s">
@@ -4799,7 +4894,7 @@
         <v>67</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>69</v>
@@ -4836,7 +4931,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P12" s="25" t="s">
@@ -4846,18 +4941,22 @@
         <v>6</v>
       </c>
       <c r="R12" s="24">
-        <f t="shared" si="3"/>
-        <v>864</v>
-      </c>
-      <c r="S12" s="20">
         <f t="shared" si="4"/>
         <v>864</v>
       </c>
+      <c r="S12" s="20">
+        <f t="shared" si="5"/>
+        <v>864</v>
+      </c>
       <c r="T12" s="27">
         <v>1107</v>
       </c>
-      <c r="U12" s="27"/>
-      <c r="V12" s="27"/>
+      <c r="U12" s="39">
+        <v>0.34</v>
+      </c>
+      <c r="V12" s="40">
+        <v>20.2</v>
+      </c>
       <c r="W12" s="9" t="s">
         <v>56</v>
       </c>
@@ -4868,7 +4967,7 @@
         <v/>
       </c>
       <c r="AA12" s="20" t="str">
-        <f>IF(OR(S12="",Z12=""),"",S12-Z12)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB12" s="10" t="s">
@@ -4920,7 +5019,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P13" s="25" t="s">
@@ -4930,18 +5029,22 @@
         <v>2</v>
       </c>
       <c r="R13" s="24">
-        <f t="shared" si="3"/>
-        <v>288</v>
-      </c>
-      <c r="S13" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
+      <c r="S13" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
       <c r="T13" s="27">
         <v>740</v>
       </c>
-      <c r="U13" s="27"/>
-      <c r="V13" s="27"/>
+      <c r="U13" s="39">
+        <v>0.5</v>
+      </c>
+      <c r="V13" s="29">
+        <v>18</v>
+      </c>
       <c r="W13" s="9" t="s">
         <v>56</v>
       </c>
@@ -4952,7 +5055,7 @@
         <v/>
       </c>
       <c r="AA13" s="20" t="str">
-        <f>IF(OR(S13="",Z13=""),"",S13-Z13)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB13" s="10" t="s">
@@ -5004,7 +5107,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P14" s="25" t="s">
@@ -5014,18 +5117,22 @@
         <v>3</v>
       </c>
       <c r="R14" s="24">
-        <f t="shared" si="3"/>
-        <v>432</v>
-      </c>
-      <c r="S14" s="20">
         <f t="shared" si="4"/>
         <v>432</v>
       </c>
+      <c r="S14" s="20">
+        <f t="shared" si="5"/>
+        <v>432</v>
+      </c>
       <c r="T14" s="27">
         <v>865</v>
       </c>
-      <c r="U14" s="27"/>
-      <c r="V14" s="27"/>
+      <c r="U14" s="39">
+        <v>0.35</v>
+      </c>
+      <c r="V14" s="29">
+        <v>18</v>
+      </c>
       <c r="W14" s="9" t="s">
         <v>56</v>
       </c>
@@ -5036,7 +5143,7 @@
         <v/>
       </c>
       <c r="AA14" s="20" t="str">
-        <f>IF(OR(S14="",Z14=""),"",S14-Z14)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB14" s="10" t="s">
@@ -5088,7 +5195,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P15" s="25" t="s">
@@ -5098,18 +5205,22 @@
         <v>2</v>
       </c>
       <c r="R15" s="24">
-        <f t="shared" si="3"/>
-        <v>288</v>
-      </c>
-      <c r="S15" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
+      <c r="S15" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
       <c r="T15" s="27">
         <v>403</v>
       </c>
-      <c r="U15" s="27"/>
-      <c r="V15" s="27"/>
+      <c r="U15" s="37">
+        <v>0.61</v>
+      </c>
+      <c r="V15" s="38">
+        <v>19</v>
+      </c>
       <c r="W15" s="9" t="s">
         <v>30</v>
       </c>
@@ -5120,7 +5231,7 @@
         <v/>
       </c>
       <c r="AA15" s="20" t="str">
-        <f>IF(OR(S15="",Z15=""),"",S15-Z15)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB15" s="10" t="s">
@@ -5172,7 +5283,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P16" s="25" t="s">
@@ -5182,18 +5293,22 @@
         <v>1</v>
       </c>
       <c r="R16" s="24">
-        <f t="shared" si="3"/>
-        <v>144</v>
-      </c>
-      <c r="S16" s="20">
         <f t="shared" si="4"/>
         <v>144</v>
       </c>
+      <c r="S16" s="20">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
       <c r="T16" s="27">
         <v>403</v>
       </c>
-      <c r="U16" s="27"/>
-      <c r="V16" s="27"/>
+      <c r="U16" s="37">
+        <v>0.74</v>
+      </c>
+      <c r="V16" s="29">
+        <v>18</v>
+      </c>
       <c r="W16" s="9" t="s">
         <v>30</v>
       </c>
@@ -5204,7 +5319,7 @@
         <v/>
       </c>
       <c r="AA16" s="20" t="str">
-        <f>IF(OR(S16="",Z16=""),"",S16-Z16)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB16" s="10" t="s">
@@ -5256,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="O17" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P17" s="25" t="s">
@@ -5266,18 +5381,22 @@
         <v>4</v>
       </c>
       <c r="R17" s="24">
-        <f t="shared" si="3"/>
-        <v>576</v>
-      </c>
-      <c r="S17" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
+      <c r="S17" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
       <c r="T17" s="27">
         <v>1069</v>
       </c>
-      <c r="U17" s="27"/>
-      <c r="V17" s="27"/>
+      <c r="U17" s="39">
+        <v>0.52</v>
+      </c>
+      <c r="V17" s="29">
+        <v>18</v>
+      </c>
       <c r="W17" s="9" t="s">
         <v>56</v>
       </c>
@@ -5288,7 +5407,7 @@
         <v/>
       </c>
       <c r="AA17" s="20" t="str">
-        <f>IF(OR(S17="",Z17=""),"",S17-Z17)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB17" s="10" t="s">
@@ -5340,7 +5459,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P18" s="25" t="s">
@@ -5350,18 +5469,22 @@
         <v>2</v>
       </c>
       <c r="R18" s="24">
-        <f t="shared" si="3"/>
-        <v>288</v>
-      </c>
-      <c r="S18" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
+      <c r="S18" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
       <c r="T18" s="27">
         <v>854</v>
       </c>
-      <c r="U18" s="27"/>
-      <c r="V18" s="27"/>
+      <c r="U18" s="39">
+        <v>0.59</v>
+      </c>
+      <c r="V18" s="29">
+        <v>18</v>
+      </c>
       <c r="W18" s="9" t="s">
         <v>56</v>
       </c>
@@ -5372,7 +5495,7 @@
         <v/>
       </c>
       <c r="AA18" s="20" t="str">
-        <f>IF(OR(S18="",Z18=""),"",S18-Z18)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB18" s="10" t="s">
@@ -5424,7 +5547,7 @@
         <v>0</v>
       </c>
       <c r="O19" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P19" s="25" t="s">
@@ -5434,18 +5557,22 @@
         <v>6</v>
       </c>
       <c r="R19" s="24">
-        <f t="shared" si="3"/>
-        <v>864</v>
-      </c>
-      <c r="S19" s="20">
         <f t="shared" si="4"/>
         <v>864</v>
       </c>
+      <c r="S19" s="20">
+        <f t="shared" si="5"/>
+        <v>864</v>
+      </c>
       <c r="T19" s="27">
         <v>538</v>
       </c>
-      <c r="U19" s="27"/>
-      <c r="V19" s="27"/>
+      <c r="U19" s="37">
+        <v>0.41</v>
+      </c>
+      <c r="V19" s="38">
+        <v>20</v>
+      </c>
       <c r="W19" s="9" t="s">
         <v>30</v>
       </c>
@@ -5456,7 +5583,7 @@
         <v/>
       </c>
       <c r="AA19" s="20" t="str">
-        <f>IF(OR(S19="",Z19=""),"",S19-Z19)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB19" s="10" t="s">
@@ -5508,7 +5635,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P20" s="25" t="s">
@@ -5518,18 +5645,22 @@
         <v>4</v>
       </c>
       <c r="R20" s="24">
-        <f t="shared" si="3"/>
-        <v>576</v>
-      </c>
-      <c r="S20" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
+      <c r="S20" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
       <c r="T20" s="27">
         <v>1064</v>
       </c>
-      <c r="U20" s="27"/>
-      <c r="V20" s="27"/>
+      <c r="U20" s="39">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="V20" s="29">
+        <v>18</v>
+      </c>
       <c r="W20" s="9" t="s">
         <v>56</v>
       </c>
@@ -5540,7 +5671,7 @@
         <v/>
       </c>
       <c r="AA20" s="20" t="str">
-        <f>IF(OR(S20="",Z20=""),"",S20-Z20)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB20" s="10" t="s">
@@ -5592,7 +5723,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P21" s="25" t="s">
@@ -5602,18 +5733,22 @@
         <v>1</v>
       </c>
       <c r="R21" s="24">
-        <f t="shared" si="3"/>
-        <v>144</v>
-      </c>
-      <c r="S21" s="20">
         <f t="shared" si="4"/>
         <v>144</v>
       </c>
+      <c r="S21" s="20">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
       <c r="T21" s="27">
         <v>538</v>
       </c>
-      <c r="U21" s="27"/>
-      <c r="V21" s="27"/>
+      <c r="U21" s="39">
+        <v>0.49</v>
+      </c>
+      <c r="V21" s="29">
+        <v>18</v>
+      </c>
       <c r="W21" s="9" t="s">
         <v>56</v>
       </c>
@@ -5624,7 +5759,7 @@
         <v/>
       </c>
       <c r="AA21" s="20" t="str">
-        <f>IF(OR(S21="",Z21=""),"",S21-Z21)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB21" s="10" t="s">
@@ -5676,7 +5811,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P22" s="25" t="s">
@@ -5686,18 +5821,22 @@
         <v>4</v>
       </c>
       <c r="R22" s="24">
-        <f t="shared" si="3"/>
-        <v>576</v>
-      </c>
-      <c r="S22" s="20">
         <f t="shared" si="4"/>
         <v>576</v>
       </c>
+      <c r="S22" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
       <c r="T22" s="27">
         <v>1133</v>
       </c>
-      <c r="U22" s="27"/>
-      <c r="V22" s="27"/>
+      <c r="U22" s="39">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="V22" s="29">
+        <v>18</v>
+      </c>
       <c r="W22" s="9" t="s">
         <v>56</v>
       </c>
@@ -5708,7 +5847,7 @@
         <v/>
       </c>
       <c r="AA22" s="20" t="str">
-        <f>IF(OR(S22="",Z22=""),"",S22-Z22)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB22" s="10" t="s">
@@ -5760,7 +5899,7 @@
         <v>0</v>
       </c>
       <c r="O23" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P23" s="25" t="s">
@@ -5770,18 +5909,22 @@
         <v>2</v>
       </c>
       <c r="R23" s="24">
-        <f t="shared" si="3"/>
-        <v>288</v>
-      </c>
-      <c r="S23" s="20">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
+      <c r="S23" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
       <c r="T23" s="27">
         <v>900</v>
       </c>
-      <c r="U23" s="27"/>
-      <c r="V23" s="27"/>
+      <c r="U23" s="39">
+        <v>0.54</v>
+      </c>
+      <c r="V23" s="29">
+        <v>18</v>
+      </c>
       <c r="W23" s="9" t="s">
         <v>56</v>
       </c>
@@ -5792,7 +5935,7 @@
         <v/>
       </c>
       <c r="AA23" s="20" t="str">
-        <f>IF(OR(S23="",Z23=""),"",S23-Z23)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB23" s="10" t="s">
@@ -5854,7 +5997,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S24" s="20">
@@ -5864,7 +6007,7 @@
       <c r="T24" s="29">
         <v>229</v>
       </c>
-      <c r="U24" s="29"/>
+      <c r="U24" s="37"/>
       <c r="V24" s="29"/>
       <c r="W24" s="9" t="s">
         <v>30</v>
@@ -5876,7 +6019,7 @@
         <v/>
       </c>
       <c r="AA24" s="20" t="str">
-        <f>IF(OR(S24="",Z24=""),"",S24-Z24)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB24" s="10" t="s">
@@ -5903,7 +6046,7 @@
         <v>40</v>
       </c>
       <c r="G25" s="18">
-        <f t="shared" ref="G25" si="7">ROUND(F25/0.8,0)</f>
+        <f t="shared" ref="G25" si="8">ROUND(F25/0.8,0)</f>
         <v>50</v>
       </c>
       <c r="H25" s="8" t="s">
@@ -5928,7 +6071,7 @@
         <v>2</v>
       </c>
       <c r="O25" s="20">
-        <f t="shared" ref="O25:O38" si="8">72*N25</f>
+        <f t="shared" ref="O25:O38" si="9">72*N25</f>
         <v>144</v>
       </c>
       <c r="P25" s="25" t="s">
@@ -5938,17 +6081,17 @@
         <v>0</v>
       </c>
       <c r="R25" s="24">
-        <f t="shared" ref="R25:R33" si="9">4*36*Q25</f>
+        <f t="shared" ref="R25:R33" si="10">4*36*Q25</f>
         <v>0</v>
       </c>
       <c r="S25" s="20">
-        <f t="shared" ref="S25:S38" si="10">O25</f>
+        <f t="shared" ref="S25:S38" si="11">O25</f>
         <v>144</v>
       </c>
       <c r="T25" s="29">
         <v>168</v>
       </c>
-      <c r="U25" s="29"/>
+      <c r="U25" s="37"/>
       <c r="V25" s="29"/>
       <c r="W25" s="9" t="s">
         <v>30</v>
@@ -5956,11 +6099,11 @@
       <c r="X25" s="9"/>
       <c r="Y25" s="20"/>
       <c r="Z25" s="20" t="str">
-        <f t="shared" ref="Z25" si="11">IF(OR(X25="",Y25=""),"",X25*Y25)</f>
+        <f t="shared" ref="Z25" si="12">IF(OR(X25="",Y25=""),"",X25*Y25)</f>
         <v/>
       </c>
       <c r="AA25" s="20" t="str">
-        <f>IF(OR(S25="",Z25=""),"",S25-Z25)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB25" s="10" t="s">
@@ -5987,7 +6130,7 @@
         <v>80</v>
       </c>
       <c r="G26" s="18">
-        <f t="shared" ref="G26:G38" si="12">ROUND(F26/0.8,0)</f>
+        <f t="shared" ref="G26:G38" si="13">ROUND(F26/0.8,0)</f>
         <v>100</v>
       </c>
       <c r="H26" s="8" t="s">
@@ -6012,7 +6155,7 @@
         <v>0</v>
       </c>
       <c r="O26" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="P26" s="25" t="s">
@@ -6022,17 +6165,17 @@
         <v>0</v>
       </c>
       <c r="R26" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S26" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="T26" s="29">
         <v>0</v>
       </c>
-      <c r="U26" s="29"/>
+      <c r="U26" s="37"/>
       <c r="V26" s="29"/>
       <c r="W26" s="9" t="s">
         <v>30</v>
@@ -6040,11 +6183,11 @@
       <c r="X26" s="9"/>
       <c r="Y26" s="20"/>
       <c r="Z26" s="20" t="str">
-        <f t="shared" ref="Z26:Z38" si="13">IF(OR(X26="",Y26=""),"",X26*Y26)</f>
+        <f t="shared" ref="Z26:Z38" si="14">IF(OR(X26="",Y26=""),"",X26*Y26)</f>
         <v/>
       </c>
       <c r="AA26" s="20" t="str">
-        <f>IF(OR(S26="",Z26=""),"",S26-Z26)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB26" s="10" t="s">
@@ -6071,7 +6214,7 @@
         <v>320</v>
       </c>
       <c r="G27" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H27" s="8" t="s">
@@ -6106,17 +6249,17 @@
         <v>0</v>
       </c>
       <c r="R27" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S27" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>288</v>
       </c>
       <c r="T27" s="29">
         <v>291</v>
       </c>
-      <c r="U27" s="29"/>
+      <c r="U27" s="37"/>
       <c r="V27" s="29"/>
       <c r="W27" s="9" t="s">
         <v>56</v>
@@ -6124,11 +6267,11 @@
       <c r="X27" s="9"/>
       <c r="Y27" s="20"/>
       <c r="Z27" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA27" s="20" t="str">
-        <f>IF(OR(S27="",Z27=""),"",S27-Z27)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB27" s="10" t="s">
@@ -6155,7 +6298,7 @@
         <v>320</v>
       </c>
       <c r="G28" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H28" s="8" t="s">
@@ -6180,7 +6323,7 @@
         <v>4</v>
       </c>
       <c r="O28" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>288</v>
       </c>
       <c r="P28" s="25" t="s">
@@ -6190,17 +6333,17 @@
         <v>0</v>
       </c>
       <c r="R28" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S28" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>288</v>
       </c>
       <c r="T28" s="29">
         <v>384</v>
       </c>
-      <c r="U28" s="29"/>
+      <c r="U28" s="37"/>
       <c r="V28" s="29"/>
       <c r="W28" s="9" t="s">
         <v>56</v>
@@ -6208,11 +6351,11 @@
       <c r="X28" s="9"/>
       <c r="Y28" s="20"/>
       <c r="Z28" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA28" s="20" t="str">
-        <f>IF(OR(S28="",Z28=""),"",S28-Z28)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB28" s="10" t="s">
@@ -6239,7 +6382,7 @@
         <v>320</v>
       </c>
       <c r="G29" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H29" s="8" t="s">
@@ -6264,7 +6407,7 @@
         <v>5</v>
       </c>
       <c r="O29" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>360</v>
       </c>
       <c r="P29" s="25" t="s">
@@ -6274,17 +6417,17 @@
         <v>0</v>
       </c>
       <c r="R29" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S29" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>360</v>
       </c>
       <c r="T29" s="29">
         <v>375</v>
       </c>
-      <c r="U29" s="29"/>
+      <c r="U29" s="37"/>
       <c r="V29" s="29"/>
       <c r="W29" s="9" t="s">
         <v>56</v>
@@ -6292,11 +6435,11 @@
       <c r="X29" s="9"/>
       <c r="Y29" s="20"/>
       <c r="Z29" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA29" s="20" t="str">
-        <f>IF(OR(S29="",Z29=""),"",S29-Z29)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB29" s="10" t="s">
@@ -6323,7 +6466,7 @@
         <v>160</v>
       </c>
       <c r="G30" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>200</v>
       </c>
       <c r="H30" s="8" t="s">
@@ -6348,7 +6491,7 @@
         <v>7</v>
       </c>
       <c r="O30" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>504</v>
       </c>
       <c r="P30" s="25" t="s">
@@ -6358,17 +6501,17 @@
         <v>0</v>
       </c>
       <c r="R30" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S30" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>504</v>
       </c>
       <c r="T30" s="29">
         <v>316</v>
       </c>
-      <c r="U30" s="29"/>
+      <c r="U30" s="37"/>
       <c r="V30" s="29"/>
       <c r="W30" s="9" t="s">
         <v>30</v>
@@ -6376,11 +6519,11 @@
       <c r="X30" s="9"/>
       <c r="Y30" s="20"/>
       <c r="Z30" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA30" s="20" t="str">
-        <f>IF(OR(S30="",Z30=""),"",S30-Z30)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB30" s="10" t="s">
@@ -6407,7 +6550,7 @@
         <v>320</v>
       </c>
       <c r="G31" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H31" s="8" t="s">
@@ -6432,7 +6575,7 @@
         <v>9</v>
       </c>
       <c r="O31" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>648</v>
       </c>
       <c r="P31" s="25" t="s">
@@ -6442,17 +6585,17 @@
         <v>0</v>
       </c>
       <c r="R31" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S31" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>648</v>
       </c>
       <c r="T31" s="29">
         <v>476</v>
       </c>
-      <c r="U31" s="29"/>
+      <c r="U31" s="37"/>
       <c r="V31" s="29"/>
       <c r="W31" s="9" t="s">
         <v>56</v>
@@ -6460,11 +6603,11 @@
       <c r="X31" s="9"/>
       <c r="Y31" s="20"/>
       <c r="Z31" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA31" s="20" t="str">
-        <f>IF(OR(S31="",Z31=""),"",S31-Z31)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB31" s="10" t="s">
@@ -6491,7 +6634,7 @@
         <v>320</v>
       </c>
       <c r="G32" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H32" s="8" t="s">
@@ -6516,7 +6659,7 @@
         <v>6</v>
       </c>
       <c r="O32" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>432</v>
       </c>
       <c r="P32" s="25" t="s">
@@ -6526,17 +6669,17 @@
         <v>0</v>
       </c>
       <c r="R32" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S32" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>432</v>
       </c>
       <c r="T32" s="29">
         <v>552</v>
       </c>
-      <c r="U32" s="29"/>
+      <c r="U32" s="37"/>
       <c r="V32" s="29"/>
       <c r="W32" s="9" t="s">
         <v>56</v>
@@ -6544,11 +6687,11 @@
       <c r="X32" s="9"/>
       <c r="Y32" s="20"/>
       <c r="Z32" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA32" s="20" t="str">
-        <f>IF(OR(S32="",Z32=""),"",S32-Z32)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB32" s="10" t="s">
@@ -6575,7 +6718,7 @@
         <v>80</v>
       </c>
       <c r="G33" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>100</v>
       </c>
       <c r="H33" s="8" t="s">
@@ -6600,7 +6743,7 @@
         <v>2</v>
       </c>
       <c r="O33" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>144</v>
       </c>
       <c r="P33" s="25" t="s">
@@ -6610,17 +6753,17 @@
         <v>0</v>
       </c>
       <c r="R33" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S33" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>144</v>
       </c>
       <c r="T33" s="29">
         <v>227</v>
       </c>
-      <c r="U33" s="29"/>
+      <c r="U33" s="37"/>
       <c r="V33" s="29"/>
       <c r="W33" s="9" t="s">
         <v>30</v>
@@ -6628,11 +6771,11 @@
       <c r="X33" s="9"/>
       <c r="Y33" s="20"/>
       <c r="Z33" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA33" s="20" t="str">
-        <f>IF(OR(S33="",Z33=""),"",S33-Z33)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB33" s="10" t="s">
@@ -6659,7 +6802,7 @@
         <v>320</v>
       </c>
       <c r="G34" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H34" s="8" t="s">
@@ -6684,7 +6827,7 @@
         <v>9</v>
       </c>
       <c r="O34" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>648</v>
       </c>
       <c r="P34" s="25" t="s">
@@ -6698,13 +6841,13 @@
         <v>0</v>
       </c>
       <c r="S34" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>648</v>
       </c>
       <c r="T34" s="29">
         <v>676</v>
       </c>
-      <c r="U34" s="29"/>
+      <c r="U34" s="37"/>
       <c r="V34" s="29"/>
       <c r="W34" s="9" t="s">
         <v>56</v>
@@ -6712,11 +6855,11 @@
       <c r="X34" s="9"/>
       <c r="Y34" s="20"/>
       <c r="Z34" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA34" s="20" t="str">
-        <f>IF(OR(S34="",Z34=""),"",S34-Z34)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB34" s="10" t="s">
@@ -6743,7 +6886,7 @@
         <v>80</v>
       </c>
       <c r="G35" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>100</v>
       </c>
       <c r="H35" s="8" t="s">
@@ -6778,7 +6921,7 @@
         <v>0</v>
       </c>
       <c r="R35" s="24">
-        <f t="shared" ref="R35:R38" si="14">4*36*Q35</f>
+        <f t="shared" ref="R35:R38" si="15">4*36*Q35</f>
         <v>0</v>
       </c>
       <c r="S35" s="20">
@@ -6788,7 +6931,7 @@
       <c r="T35" s="29">
         <v>273</v>
       </c>
-      <c r="U35" s="29"/>
+      <c r="U35" s="37"/>
       <c r="V35" s="29"/>
       <c r="W35" s="9" t="s">
         <v>30</v>
@@ -6796,11 +6939,11 @@
       <c r="X35" s="9"/>
       <c r="Y35" s="20"/>
       <c r="Z35" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA35" s="20" t="str">
-        <f>IF(OR(S35="",Z35=""),"",S35-Z35)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB35" s="10" t="s">
@@ -6827,7 +6970,7 @@
         <v>320</v>
       </c>
       <c r="G36" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H36" s="8" t="s">
@@ -6852,7 +6995,7 @@
         <v>8</v>
       </c>
       <c r="O36" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>576</v>
       </c>
       <c r="P36" s="25" t="s">
@@ -6862,17 +7005,17 @@
         <v>0</v>
       </c>
       <c r="R36" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="S36" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>576</v>
       </c>
       <c r="T36" s="29">
         <v>622</v>
       </c>
-      <c r="U36" s="29"/>
+      <c r="U36" s="37"/>
       <c r="V36" s="29"/>
       <c r="W36" s="9" t="s">
         <v>56</v>
@@ -6880,11 +7023,11 @@
       <c r="X36" s="9"/>
       <c r="Y36" s="20"/>
       <c r="Z36" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA36" s="20" t="str">
-        <f>IF(OR(S36="",Z36=""),"",S36-Z36)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB36" s="10" t="s">
@@ -6911,13 +7054,13 @@
         <v>80</v>
       </c>
       <c r="G37" s="18">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>100</v>
       </c>
       <c r="H37" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="I37" s="34" t="s">
+      <c r="I37" s="33" t="s">
         <v>196</v>
       </c>
       <c r="J37" s="8" t="s">
@@ -6936,7 +7079,7 @@
         <v>1</v>
       </c>
       <c r="O37" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>72</v>
       </c>
       <c r="P37" s="25" t="s">
@@ -6946,17 +7089,17 @@
         <v>0</v>
       </c>
       <c r="R37" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="S37" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>72</v>
       </c>
       <c r="T37" s="29">
         <v>136</v>
       </c>
-      <c r="U37" s="29"/>
+      <c r="U37" s="37"/>
       <c r="V37" s="29"/>
       <c r="W37" s="9" t="s">
         <v>30</v>
@@ -6964,11 +7107,11 @@
       <c r="X37" s="9"/>
       <c r="Y37" s="20"/>
       <c r="Z37" s="20" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA37" s="20" t="str">
-        <f>IF(OR(S37="",Z37=""),"",S37-Z37)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB37" s="10" t="s">
@@ -6995,13 +7138,13 @@
         <v>320</v>
       </c>
       <c r="G38" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>400</v>
       </c>
       <c r="H38" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="I38" s="34" t="s">
+      <c r="I38" s="33" t="s">
         <v>195</v>
       </c>
       <c r="J38" s="13" t="s">
@@ -7020,7 +7163,7 @@
         <v>8</v>
       </c>
       <c r="O38" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>576</v>
       </c>
       <c r="P38" s="25" t="s">
@@ -7030,17 +7173,17 @@
         <v>0</v>
       </c>
       <c r="R38" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="S38" s="20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>576</v>
       </c>
       <c r="T38" s="29">
         <v>458</v>
       </c>
-      <c r="U38" s="29"/>
+      <c r="U38" s="37"/>
       <c r="V38" s="29"/>
       <c r="W38" s="14" t="s">
         <v>56</v>
@@ -7048,11 +7191,11 @@
       <c r="X38" s="14"/>
       <c r="Y38" s="21"/>
       <c r="Z38" s="21" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="AA38" s="21" t="str">
-        <f>IF(OR(S38="",Z38=""),"",S38-Z38)</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="AB38" s="15" t="s">
@@ -7074,19 +7217,19 @@
     <mergeCell ref="A1:Z1"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="T4:V23 U25:V25">
-    <cfRule type="expression" dxfId="3" priority="3">
+  <conditionalFormatting sqref="T4:T23">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>$T4&gt;=$F4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="4" priority="4">
       <formula>$T4&lt;$F4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T25">
-    <cfRule type="expression" dxfId="1" priority="1">
+  <conditionalFormatting sqref="T25:V25">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>$T25&gt;=$F25</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>$T25&lt;$F25</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7098,7 +7241,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="8.8125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
@@ -7106,19 +7249,19 @@
     <col min="6" max="8" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20.65">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:8" ht="20.25">
+      <c r="A1" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-    </row>
-    <row r="2" spans="1:8" ht="27.75">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+    </row>
+    <row r="2" spans="1:8" ht="30">
       <c r="A2" s="1" t="s">
         <v>148</v>
       </c>
@@ -7144,7 +7287,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="27">
+    <row r="3" spans="1:8" ht="28.5">
       <c r="A3" s="2" t="s">
         <v>69</v>
       </c>
@@ -7171,7 +7314,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="27">
+    <row r="4" spans="1:8" ht="28.5">
       <c r="A4" s="2" t="s">
         <v>158</v>
       </c>
@@ -7333,7 +7476,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="27">
+    <row r="10" spans="1:8" ht="28.5">
       <c r="A10" s="2" t="s">
         <v>174</v>
       </c>

</xml_diff>

<commit_message>
Updated Building B First Floor report. Added uniformity and glare at 1.2m
</commit_message>
<xml_diff>
--- a/excel/Building A B and carpark Lighting New.xlsx
+++ b/excel/Building A B and carpark Lighting New.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F835CACE-7537-4F06-AA1F-FE3CCD4C11F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23E3571-EFBD-4E3D-B9E5-7C3E2498E5AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="201">
   <si>
     <t>Building A — Lighting Place Schedule</t>
   </si>
@@ -633,12 +633,21 @@
   </si>
   <si>
     <t>Glare (UGGR)</t>
+  </si>
+  <si>
+    <t>Uniformity (Uo) in x-direction (g1)</t>
+  </si>
+  <si>
+    <t>Office (CAD)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="0.0"/>
+  </numFmts>
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -679,7 +688,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -736,6 +745,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -820,7 +847,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -928,6 +955,27 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="3" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -937,7 +985,35 @@
     <cellStyle name="Normal 5" xfId="4" xr:uid="{ED6D2035-F9DA-4B1D-B2ED-B5DB87628F59}"/>
     <cellStyle name="Normal 6" xfId="5" xr:uid="{FCC80704-4661-421C-AAE8-B6CB6410940C}"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3882,10 +3958,10 @@
     <mergeCell ref="A1:W1"/>
   </mergeCells>
   <conditionalFormatting sqref="T4:V36">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>$T4&lt;$F4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>$T4&gt;=$F4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3904,15 +3980,15 @@
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="7" width="14" customWidth="1"/>
     <col min="8" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="34" customWidth="1"/>
-    <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="34" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="15.6875" customWidth="1"/>
-    <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="20" width="14" customWidth="1"/>
+    <col min="10" max="10" width="34" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="30" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="34" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="22" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="12" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="14" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="15.6875" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="12" hidden="1" customWidth="1"/>
+    <col min="19" max="20" width="14" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="24" customWidth="1"/>
     <col min="22" max="23" width="12" customWidth="1"/>
     <col min="24" max="25" width="14" customWidth="1"/>
@@ -4011,7 +4087,7 @@
         <v>185</v>
       </c>
       <c r="U2" s="26" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="V2" s="26" t="s">
         <v>198</v>
@@ -5864,8 +5940,10 @@
       <c r="T24" s="29">
         <v>229</v>
       </c>
-      <c r="U24" s="29"/>
-      <c r="V24" s="29"/>
+      <c r="U24" s="38">
+        <v>0.93</v>
+      </c>
+      <c r="V24" s="41"/>
       <c r="W24" s="9" t="s">
         <v>30</v>
       </c>
@@ -5948,8 +6026,10 @@
       <c r="T25" s="29">
         <v>168</v>
       </c>
-      <c r="U25" s="29"/>
-      <c r="V25" s="29"/>
+      <c r="U25" s="42">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V25" s="41"/>
       <c r="W25" s="9" t="s">
         <v>30</v>
       </c>
@@ -6032,8 +6112,10 @@
       <c r="T26" s="29">
         <v>0</v>
       </c>
-      <c r="U26" s="29"/>
-      <c r="V26" s="29"/>
+      <c r="U26" s="40">
+        <v>0</v>
+      </c>
+      <c r="V26" s="39"/>
       <c r="W26" s="9" t="s">
         <v>30</v>
       </c>
@@ -6116,8 +6198,12 @@
       <c r="T27" s="29">
         <v>291</v>
       </c>
-      <c r="U27" s="29"/>
-      <c r="V27" s="29"/>
+      <c r="U27" s="42">
+        <v>0.67</v>
+      </c>
+      <c r="V27" s="43">
+        <v>22</v>
+      </c>
       <c r="W27" s="9" t="s">
         <v>56</v>
       </c>
@@ -6200,8 +6286,12 @@
       <c r="T28" s="29">
         <v>384</v>
       </c>
-      <c r="U28" s="29"/>
-      <c r="V28" s="29"/>
+      <c r="U28" s="38">
+        <v>0.77</v>
+      </c>
+      <c r="V28" s="43">
+        <v>20.8</v>
+      </c>
       <c r="W28" s="9" t="s">
         <v>56</v>
       </c>
@@ -6284,8 +6374,12 @@
       <c r="T29" s="29">
         <v>375</v>
       </c>
-      <c r="U29" s="29"/>
-      <c r="V29" s="29"/>
+      <c r="U29" s="42">
+        <v>0.59</v>
+      </c>
+      <c r="V29" s="43">
+        <v>22.6</v>
+      </c>
       <c r="W29" s="9" t="s">
         <v>56</v>
       </c>
@@ -6368,8 +6462,12 @@
       <c r="T30" s="29">
         <v>316</v>
       </c>
-      <c r="U30" s="29"/>
-      <c r="V30" s="29"/>
+      <c r="U30" s="38">
+        <v>0.62</v>
+      </c>
+      <c r="V30" s="43">
+        <v>25.1</v>
+      </c>
       <c r="W30" s="9" t="s">
         <v>30</v>
       </c>
@@ -6395,7 +6493,7 @@
         <v>89</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>68</v>
+        <v>200</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>69</v>
@@ -6452,8 +6550,12 @@
       <c r="T31" s="29">
         <v>476</v>
       </c>
-      <c r="U31" s="29"/>
-      <c r="V31" s="29"/>
+      <c r="U31" s="42">
+        <v>0.66</v>
+      </c>
+      <c r="V31" s="43">
+        <v>21.4</v>
+      </c>
       <c r="W31" s="9" t="s">
         <v>56</v>
       </c>
@@ -6536,8 +6638,12 @@
       <c r="T32" s="29">
         <v>552</v>
       </c>
-      <c r="U32" s="29"/>
-      <c r="V32" s="29"/>
+      <c r="U32" s="38">
+        <v>0.72</v>
+      </c>
+      <c r="V32" s="37">
+        <v>18.5</v>
+      </c>
       <c r="W32" s="9" t="s">
         <v>56</v>
       </c>
@@ -6620,8 +6726,12 @@
       <c r="T33" s="29">
         <v>227</v>
       </c>
-      <c r="U33" s="29"/>
-      <c r="V33" s="29"/>
+      <c r="U33" s="38">
+        <v>0.87</v>
+      </c>
+      <c r="V33" s="37">
+        <v>17.5</v>
+      </c>
       <c r="W33" s="9" t="s">
         <v>30</v>
       </c>
@@ -6704,8 +6814,12 @@
       <c r="T34" s="29">
         <v>676</v>
       </c>
-      <c r="U34" s="29"/>
-      <c r="V34" s="29"/>
+      <c r="U34" s="42">
+        <v>0.68</v>
+      </c>
+      <c r="V34" s="43">
+        <v>21.5</v>
+      </c>
       <c r="W34" s="9" t="s">
         <v>56</v>
       </c>
@@ -6788,8 +6902,12 @@
       <c r="T35" s="29">
         <v>273</v>
       </c>
-      <c r="U35" s="29"/>
-      <c r="V35" s="29"/>
+      <c r="U35" s="38">
+        <v>0.66</v>
+      </c>
+      <c r="V35" s="37">
+        <v>21.1</v>
+      </c>
       <c r="W35" s="9" t="s">
         <v>30</v>
       </c>
@@ -6872,8 +6990,12 @@
       <c r="T36" s="29">
         <v>622</v>
       </c>
-      <c r="U36" s="29"/>
-      <c r="V36" s="29"/>
+      <c r="U36" s="38">
+        <v>0.7</v>
+      </c>
+      <c r="V36" s="37">
+        <v>18.7</v>
+      </c>
       <c r="W36" s="9" t="s">
         <v>56</v>
       </c>
@@ -6956,8 +7078,12 @@
       <c r="T37" s="29">
         <v>136</v>
       </c>
-      <c r="U37" s="29"/>
-      <c r="V37" s="29"/>
+      <c r="U37" s="38">
+        <v>0.76</v>
+      </c>
+      <c r="V37" s="37">
+        <v>11.9</v>
+      </c>
       <c r="W37" s="9" t="s">
         <v>30</v>
       </c>
@@ -7040,8 +7166,12 @@
       <c r="T38" s="29">
         <v>458</v>
       </c>
-      <c r="U38" s="29"/>
-      <c r="V38" s="29"/>
+      <c r="U38" s="42">
+        <v>0.62</v>
+      </c>
+      <c r="V38" s="43">
+        <v>20.8</v>
+      </c>
       <c r="W38" s="14" t="s">
         <v>56</v>
       </c>
@@ -7074,19 +7204,19 @@
     <mergeCell ref="A1:Z1"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="T4:V23 U25:V25">
-    <cfRule type="expression" dxfId="3" priority="3">
+  <conditionalFormatting sqref="T4:V23">
+    <cfRule type="expression" dxfId="7" priority="3">
       <formula>$T4&gt;=$F4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="6" priority="4">
       <formula>$T4&lt;$F4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T25">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$T25&gt;=$F25</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$T25&lt;$F25</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Actually updated Building B First Floor Report.
</commit_message>
<xml_diff>
--- a/excel/Building A B and carpark Lighting New.xlsx
+++ b/excel/Building A B and carpark Lighting New.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\Alpha_Design_17\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0375D266-8CB6-4F37-B239-34A3C4DA439C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552230D9-DEFF-44A5-950C-B17A023E316B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="212">
   <si>
     <t>Building A — Lighting Place Schedule</t>
   </si>
@@ -658,6 +658,21 @@
   </si>
   <si>
     <t>&lt;= 19</t>
+  </si>
+  <si>
+    <t>Luminaire</t>
+  </si>
+  <si>
+    <t>Suspension</t>
+  </si>
+  <si>
+    <t>2.8m</t>
+  </si>
+  <si>
+    <t>ETAP R3111/LEDN445DX1 x 9</t>
+  </si>
+  <si>
+    <t>3.0m</t>
   </si>
 </sst>
 </file>
@@ -866,7 +881,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -996,6 +1011,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -7220,7 +7238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF39E06F-3BD1-49F8-AE29-EAEE385292C4}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="3" max="3" width="11.875" customWidth="1"/>
@@ -7228,11 +7246,13 @@
     <col min="5" max="5" width="14.0625" customWidth="1"/>
     <col min="6" max="6" width="16.25" customWidth="1"/>
     <col min="7" max="7" width="19.5" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="18.4375" customWidth="1"/>
+    <col min="9" max="9" width="18.8125" customWidth="1"/>
+    <col min="10" max="10" width="17.8125" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="18.4375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.75">
+    <row r="1" spans="1:13" ht="27.75">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -7258,16 +7278,22 @@
         <v>201</v>
       </c>
       <c r="I1" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="J1" s="26" t="s">
+        <v>208</v>
+      </c>
+      <c r="K1" s="26" t="s">
         <v>204</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="L1" s="26" t="s">
         <v>205</v>
       </c>
-      <c r="K1" s="26" t="s">
+      <c r="M1" s="26" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:13">
       <c r="A2" s="6" t="s">
         <v>78</v>
       </c>
@@ -7289,14 +7315,14 @@
       <c r="G2" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="I2" s="42">
+      <c r="K2" s="42">
         <v>307</v>
       </c>
-      <c r="J2" s="42">
+      <c r="L2" s="42">
         <v>0.93</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="25.5">
+    <row r="3" spans="1:13" ht="25.5">
       <c r="A3" s="6" t="s">
         <v>78</v>
       </c>
@@ -7318,14 +7344,14 @@
       <c r="G3" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="I3" s="42">
+      <c r="K3" s="42">
         <v>199</v>
       </c>
-      <c r="J3" s="43">
+      <c r="L3" s="43">
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="25.5">
+    <row r="4" spans="1:13" ht="25.5">
       <c r="A4" s="6" t="s">
         <v>78</v>
       </c>
@@ -7345,10 +7371,10 @@
         <v>80</v>
       </c>
       <c r="G4" s="8"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="K4" s="42"/>
+      <c r="L4" s="42"/>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="6" t="s">
         <v>78</v>
       </c>
@@ -7370,14 +7396,14 @@
       <c r="G5" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="I5" s="42">
+      <c r="K5" s="42">
         <v>367</v>
       </c>
-      <c r="J5" s="42">
+      <c r="L5" s="42">
         <v>0.65</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:13">
       <c r="A6" s="6" t="s">
         <v>78</v>
       </c>
@@ -7399,14 +7425,14 @@
       <c r="G6" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="42">
+      <c r="K6" s="42">
         <v>494</v>
       </c>
-      <c r="J6" s="42">
+      <c r="L6" s="42">
         <v>0.73</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="25.5">
+    <row r="7" spans="1:13" ht="25.5">
       <c r="A7" s="6" t="s">
         <v>78</v>
       </c>
@@ -7428,17 +7454,14 @@
       <c r="G7" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="H7" t="s">
-        <v>206</v>
-      </c>
-      <c r="I7" s="42">
+      <c r="K7" s="42">
         <v>481</v>
       </c>
-      <c r="J7" s="42">
+      <c r="L7" s="42">
         <v>0.62</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="25.5">
+    <row r="8" spans="1:13" ht="25.5">
       <c r="A8" s="6" t="s">
         <v>78</v>
       </c>
@@ -7460,14 +7483,20 @@
       <c r="G8" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="I8" s="42">
+      <c r="I8" t="s">
+        <v>210</v>
+      </c>
+      <c r="J8" t="s">
+        <v>211</v>
+      </c>
+      <c r="K8" s="42">
         <v>391</v>
       </c>
-      <c r="J8" s="42">
+      <c r="L8" s="42">
         <v>0.6</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="25.5">
+    <row r="9" spans="1:13" ht="40.5">
       <c r="A9" s="6" t="s">
         <v>78</v>
       </c>
@@ -7492,17 +7521,23 @@
       <c r="H9" t="s">
         <v>206</v>
       </c>
-      <c r="I9" s="42">
+      <c r="I9" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="J9" t="s">
+        <v>209</v>
+      </c>
+      <c r="K9" s="42">
         <v>588</v>
       </c>
-      <c r="J9" s="42">
+      <c r="L9" s="42">
         <v>0.66</v>
       </c>
-      <c r="K9" s="43">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+      <c r="M9" s="42">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="6" t="s">
         <v>78</v>
       </c>
@@ -7524,14 +7559,14 @@
       <c r="G10" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="I10" s="42">
+      <c r="K10" s="42">
         <v>709</v>
       </c>
-      <c r="J10" s="42">
+      <c r="L10" s="42">
         <v>0.74</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:13">
       <c r="A11" s="6" t="s">
         <v>78</v>
       </c>
@@ -7553,14 +7588,14 @@
       <c r="G11" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="I11" s="42">
+      <c r="K11" s="42">
         <v>296</v>
       </c>
-      <c r="J11" s="42">
+      <c r="L11" s="42">
         <v>0.86</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="25.5">
+    <row r="12" spans="1:13" ht="25.5">
       <c r="A12" s="6" t="s">
         <v>78</v>
       </c>
@@ -7582,17 +7617,14 @@
       <c r="G12" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="H12" t="s">
-        <v>206</v>
-      </c>
-      <c r="I12" s="42">
+      <c r="K12" s="42">
         <v>845</v>
       </c>
-      <c r="J12" s="42">
+      <c r="L12" s="42">
         <v>0.69</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:13">
       <c r="A13" s="6" t="s">
         <v>78</v>
       </c>
@@ -7614,14 +7646,14 @@
       <c r="G13" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="I13" s="42">
+      <c r="K13" s="42">
         <v>350</v>
       </c>
-      <c r="J13" s="42">
+      <c r="L13" s="42">
         <v>0.69</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="25.5">
+    <row r="14" spans="1:13" ht="25.5">
       <c r="A14" s="6" t="s">
         <v>78</v>
       </c>
@@ -7643,17 +7675,14 @@
       <c r="G14" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="H14" t="s">
-        <v>206</v>
-      </c>
-      <c r="I14" s="42">
+      <c r="K14" s="42">
         <v>785</v>
       </c>
-      <c r="J14" s="42">
+      <c r="L14" s="42">
         <v>0.72</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="25.5">
+    <row r="15" spans="1:13" ht="25.5">
       <c r="A15" s="6" t="s">
         <v>78</v>
       </c>
@@ -7675,14 +7704,14 @@
       <c r="G15" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="I15" s="42">
+      <c r="K15" s="42">
         <v>196</v>
       </c>
-      <c r="J15" s="42">
+      <c r="L15" s="42">
         <v>0.63</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:13">
       <c r="A16" s="11" t="s">
         <v>78</v>
       </c>
@@ -7704,16 +7733,17 @@
       <c r="G16" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="I16" s="42">
+      <c r="K16" s="42">
         <v>569</v>
       </c>
-      <c r="J16" s="42">
+      <c r="L16" s="42">
         <v>0.93</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>